<commit_message>
final update for the website
</commit_message>
<xml_diff>
--- a/data/all-products.xlsx
+++ b/data/all-products.xlsx
@@ -12918,10 +12918,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N236" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-harmonia-oak-tactus-nougat-1751347.jpg</v>
       </c>
       <c r="O236" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-harmonia-oak-tactus-nougat-1751347.jpg</v>
       </c>
       <c r="P236" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-harmonia-oak-tactus-nougat-1751347</v>
@@ -12971,10 +12971,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N237" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-harmonia-oak-favo-brunet-1751346.jpg</v>
       </c>
       <c r="O237" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-harmonia-oak-favo-brunet-1751346.jpg</v>
       </c>
       <c r="P237" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-harmonia-oak-favo-brunet-1751346</v>
@@ -13024,10 +13024,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N238" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-harmonia-oak-sensus-acorn-1751345.jpg</v>
       </c>
       <c r="O238" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-harmonia-oak-sensus-acorn-1751345.jpg</v>
       </c>
       <c r="P238" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-harmonia-oak-sensus-acorn-1751345</v>
@@ -13077,10 +13077,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N239" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-harmonia-oak-undula-espresso-1751343.jpg</v>
       </c>
       <c r="O239" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-harmonia-oak-undula-espresso-1751343.jpg</v>
       </c>
       <c r="P239" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-harmonia-oak-undula-espresso-1751343</v>
@@ -13130,10 +13130,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N240" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-harmonia-oak-nexus-java-1751342.jpg</v>
       </c>
       <c r="O240" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-harmonia-oak-nexus-java-1751342.jpg</v>
       </c>
       <c r="P240" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-harmonia-oak-nexus-java-1751342</v>
@@ -13183,10 +13183,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N241" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-harmonia-oak-ratio-cognac-1751340.jpg</v>
       </c>
       <c r="O241" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-harmonia-oak-ratio-cognac-1751340.jpg</v>
       </c>
       <c r="P241" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-harmonia-oak-ratio-cognac-1751340</v>
@@ -13236,10 +13236,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N242" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-harmonia-oak-flecto-champagne-1751339.jpg</v>
       </c>
       <c r="O242" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-harmonia-oak-flecto-champagne-1751339.jpg</v>
       </c>
       <c r="P242" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-harmonia-oak-flecto-champagne-1751339</v>
@@ -13289,10 +13289,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N243" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-maradune-oak-kalahari-smoked-1751304.jpg</v>
       </c>
       <c r="O243" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-maradune-oak-kalahari-smoked-1751304.jpg</v>
       </c>
       <c r="P243" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-maradune-oak-kalahari-smoked-1751304</v>
@@ -13342,10 +13342,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N244" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-maradune-oak-tanami-smoked-1751303.jpg</v>
       </c>
       <c r="O244" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-maradune-oak-tanami-smoked-1751303.jpg</v>
       </c>
       <c r="P244" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-maradune-oak-tanami-smoked-1751303</v>
@@ -13395,10 +13395,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N245" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-maradune-oak-kalahari-white-1751302.jpg</v>
       </c>
       <c r="O245" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-maradune-oak-kalahari-white-1751302.jpg</v>
       </c>
       <c r="P245" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-maradune-oak-kalahari-white-1751302</v>
@@ -13448,10 +13448,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N246" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-maradune-oak-savanna-smoked-1751301.jpg</v>
       </c>
       <c r="O246" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-maradune-oak-savanna-smoked-1751301.jpg</v>
       </c>
       <c r="P246" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-maradune-oak-savanna-smoked-1751301</v>
@@ -13501,10 +13501,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N247" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-maradune-oak-savanna-smoked-grey-1751300.jpg</v>
       </c>
       <c r="O247" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-maradune-oak-savanna-smoked-grey-1751300.jpg</v>
       </c>
       <c r="P247" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-maradune-oak-savanna-smoked-grey-1751300</v>
@@ -13554,10 +13554,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N248" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-maradune-oak-savanna-limed-1751299.jpg</v>
       </c>
       <c r="O248" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-maradune-oak-savanna-limed-1751299.jpg</v>
       </c>
       <c r="P248" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-maradune-oak-savanna-limed-1751299</v>
@@ -13607,10 +13607,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N249" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-maradune-oak-tanami-1751113.jpg</v>
       </c>
       <c r="O249" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-maradune-oak-tanami-1751113.jpg</v>
       </c>
       <c r="P249" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-maradune-oak-tanami-1751113</v>
@@ -13660,10 +13660,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N250" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-maradune-oak-kalahari-1751112.jpg</v>
       </c>
       <c r="O250" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-maradune-oak-kalahari-1751112.jpg</v>
       </c>
       <c r="P250" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-maradune-oak-kalahari-1751112</v>
@@ -13713,10 +13713,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N251" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-maradune-oak-savanna-1751111.jpg</v>
       </c>
       <c r="O251" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-maradune-oak-savanna-1751111.jpg</v>
       </c>
       <c r="P251" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-maradune-oak-savanna-1751111</v>
@@ -13766,10 +13766,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N252" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-malbec-light-whitewashed-1748912.jpg</v>
       </c>
       <c r="O252" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-malbec-light-whitewashed-1748912.jpg</v>
       </c>
       <c r="P252" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-basic-11-5-oak-malbec-light-whitewashed-1748912</v>
@@ -13819,10 +13819,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N253" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-malbec-natural-1748911.jpg</v>
       </c>
       <c r="O253" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-malbec-natural-1748911.jpg</v>
       </c>
       <c r="P253" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-basic-11-5-oak-malbec-natural-1748911</v>
@@ -13872,10 +13872,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N254" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-malbec-light-whitewashed-1748909.jpg</v>
       </c>
       <c r="O254" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-malbec-light-whitewashed-1748909.jpg</v>
       </c>
       <c r="P254" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3025-oak-malbec-light-whitewashed-1748909</v>
@@ -13925,10 +13925,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N255" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-malbec-natural-1748908.jpg</v>
       </c>
       <c r="O255" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-malbec-natural-1748908.jpg</v>
       </c>
       <c r="P255" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3025-oak-malbec-natural-1748908</v>
@@ -13978,10 +13978,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N256" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-4-oak-molvina-natural-1748907.jpg</v>
       </c>
       <c r="O256" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-4-oak-molvina-natural-1748907.jpg</v>
       </c>
       <c r="P256" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-trendtime-4-oak-molvina-natural-1748907</v>
@@ -14031,10 +14031,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N257" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-4-oak-lugana-natural-1748906.jpg</v>
       </c>
       <c r="O257" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-4-oak-lugana-natural-1748906.jpg</v>
       </c>
       <c r="P257" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-trendtime-4-oak-lugana-natural-1748906</v>
@@ -14084,10 +14084,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N258" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-4-oak-lugana-light-whitewashed-1748905.jpg</v>
       </c>
       <c r="O258" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-4-oak-lugana-light-whitewashed-1748905.jpg</v>
       </c>
       <c r="P258" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-trendtime-4-oak-lugana-light-whitewashed-1748905</v>
@@ -14137,10 +14137,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N259" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-4-oak-lugana-natural-1748904.jpg</v>
       </c>
       <c r="O259" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-4-oak-lugana-natural-1748904.jpg</v>
       </c>
       <c r="P259" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-trendtime-4-oak-lugana-natural-1748904</v>
@@ -14190,10 +14190,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N260" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-chianti-natural-1748902.jpg</v>
       </c>
       <c r="O260" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-chianti-natural-1748902.jpg</v>
       </c>
       <c r="P260" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3025-oak-chianti-natural-1748902</v>
@@ -14243,10 +14243,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N261" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-chianti-light-whitewashed-1748901.jpg</v>
       </c>
       <c r="O261" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-chianti-light-whitewashed-1748901.jpg</v>
       </c>
       <c r="P261" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3025-oak-chianti-light-whitewashed-1748901</v>
@@ -14296,10 +14296,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N262" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-chianti-natural-1748900.jpg</v>
       </c>
       <c r="O262" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-chianti-natural-1748900.jpg</v>
       </c>
       <c r="P262" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3025-oak-chianti-natural-1748900</v>
@@ -14349,10 +14349,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N263" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-chianti-natural-1748899.jpg</v>
       </c>
       <c r="O263" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-chianti-natural-1748899.jpg</v>
       </c>
       <c r="P263" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-basic-11-5-oak-chianti-natural-1748899</v>
@@ -14402,10 +14402,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N264" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-chianti-light-whitewashed-1748898.jpg</v>
       </c>
       <c r="O264" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-chianti-light-whitewashed-1748898.jpg</v>
       </c>
       <c r="P264" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-basic-11-5-oak-chianti-light-whitewashed-1748898</v>
@@ -14455,10 +14455,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N265" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-chianti-natural-1748897.jpg</v>
       </c>
       <c r="O265" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-chianti-natural-1748897.jpg</v>
       </c>
       <c r="P265" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-basic-11-5-oak-chianti-natural-1748897</v>
@@ -14508,10 +14508,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N266" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-soave-natural-1748895.jpg</v>
       </c>
       <c r="O266" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-soave-natural-1748895.jpg</v>
       </c>
       <c r="P266" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-soave-natural-1748895</v>
@@ -14561,10 +14561,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N267" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-soave-white-1748894.jpg</v>
       </c>
       <c r="O267" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-soave-white-1748894.jpg</v>
       </c>
       <c r="P267" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-soave-white-1748894</v>
@@ -14614,10 +14614,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N268" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-sauvignon-light-whitewashed-1748892.jpg</v>
       </c>
       <c r="O268" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-sauvignon-light-whitewashed-1748892.jpg</v>
       </c>
       <c r="P268" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-sauvignon-light-whitewashed-1748892</v>
@@ -14667,10 +14667,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N269" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-ash-amarone-brown-1748891.jpg</v>
       </c>
       <c r="O269" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-ash-amarone-brown-1748891.jpg</v>
       </c>
       <c r="P269" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-ash-amarone-brown-1748891</v>
@@ -14720,10 +14720,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N270" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-ash-kir-white-1748890.jpg</v>
       </c>
       <c r="O270" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-ash-kir-white-1748890.jpg</v>
       </c>
       <c r="P270" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-ash-kir-white-1748890</v>
@@ -14773,10 +14773,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N271" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-brunello-brown-1748889.jpg</v>
       </c>
       <c r="O271" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-brunello-brown-1748889.jpg</v>
       </c>
       <c r="P271" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-brunello-brown-1748889</v>
@@ -14826,10 +14826,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N272" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-pinot-black-1748887.jpg</v>
       </c>
       <c r="O272" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-pinot-black-1748887.jpg</v>
       </c>
       <c r="P272" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-pinot-black-1748887</v>
@@ -14879,10 +14879,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N273" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-3-oak-chalet-grey-1748885.jpg</v>
       </c>
       <c r="O273" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-3-oak-chalet-grey-1748885.jpg</v>
       </c>
       <c r="P273" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-trendtime-3-oak-chalet-grey-1748885</v>
@@ -14932,10 +14932,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N274" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-3-oak-bardolino-natural-1748884.jpg</v>
       </c>
       <c r="O274" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-3-oak-bardolino-natural-1748884.jpg</v>
       </c>
       <c r="P274" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-trendtime-3-oak-bardolino-natural-1748884</v>
@@ -14985,10 +14985,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N275" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-3-oak-bardolino-white-1748883.jpg</v>
       </c>
       <c r="O275" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-3-oak-bardolino-white-1748883.jpg</v>
       </c>
       <c r="P275" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-trendtime-3-oak-bardolino-white-1748883</v>
@@ -15038,10 +15038,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N276" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-cortese-natural-1748881.jpg</v>
       </c>
       <c r="O276" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-cortese-natural-1748881.jpg</v>
       </c>
       <c r="P276" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3025-oak-cortese-natural-1748881</v>
@@ -15091,10 +15091,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N277" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-cortese-white-1748879.jpg</v>
       </c>
       <c r="O277" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-cortese-white-1748879.jpg</v>
       </c>
       <c r="P277" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3025-oak-cortese-white-1748879</v>
@@ -15144,10 +15144,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N278" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-10-oak-tuscan-1748490.jpg</v>
       </c>
       <c r="O278" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-10-oak-tuscan-1748490.jpg</v>
       </c>
       <c r="P278" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-trendtime-10-oak-tuscan-1748490</v>
@@ -15197,10 +15197,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N279" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-10-oak-1748487.jpg</v>
       </c>
       <c r="O279" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-10-oak-1748487.jpg</v>
       </c>
       <c r="P279" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-trendtime-10-oak-1748487</v>
@@ -15250,10 +15250,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N280" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-10-oak-terra-1748486.jpg</v>
       </c>
       <c r="O280" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-10-oak-terra-1748486.jpg</v>
       </c>
       <c r="P280" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-trendtime-10-oak-terra-1748486</v>
@@ -15303,10 +15303,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N281" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-10-oak-natur-1748484.jpg</v>
       </c>
       <c r="O281" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-10-oak-natur-1748484.jpg</v>
       </c>
       <c r="P281" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-trendtime-10-oak-natur-1748484</v>
@@ -15356,10 +15356,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N282" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-10-oak-dune-1748483.jpg</v>
       </c>
       <c r="O282" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-10-oak-dune-1748483.jpg</v>
       </c>
       <c r="P282" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-trendtime-10-oak-dune-1748483</v>
@@ -15409,10 +15409,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N283" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-10-oak-sienna-1748482.jpg</v>
       </c>
       <c r="O283" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-10-oak-sienna-1748482.jpg</v>
       </c>
       <c r="P283" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-trendtime-10-oak-sienna-1748482</v>
@@ -15462,10 +15462,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N284" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-sanded-1744433.jpg</v>
       </c>
       <c r="O284" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-sanded-1744433.jpg</v>
       </c>
       <c r="P284" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-sanded-1744433</v>
@@ -15515,10 +15515,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N285" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1744417.jpg</v>
       </c>
       <c r="O285" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1744417.jpg</v>
       </c>
       <c r="P285" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-1744417</v>
@@ -15568,10 +15568,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N286" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-brushed-1744853.jpg</v>
       </c>
       <c r="O286" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-brushed-1744853.jpg</v>
       </c>
       <c r="P286" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3025-oak-brushed-1744853</v>
@@ -15621,10 +15621,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N287" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-brushed-1744852.jpg</v>
       </c>
       <c r="O287" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-brushed-1744852.jpg</v>
       </c>
       <c r="P287" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3025-oak-brushed-1744852</v>
@@ -15674,10 +15674,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N288" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-brushed-1744851.jpg</v>
       </c>
       <c r="O288" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-brushed-1744851.jpg</v>
       </c>
       <c r="P288" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3025-oak-brushed-1744851</v>
@@ -15727,10 +15727,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N289" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-soft-texture-1744846.jpg</v>
       </c>
       <c r="O289" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-soft-texture-1744846.jpg</v>
       </c>
       <c r="P289" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3025-oak-soft-texture-1744846</v>
@@ -15780,10 +15780,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N290" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-brushed-1744854.jpg</v>
       </c>
       <c r="O290" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-brushed-1744854.jpg</v>
       </c>
       <c r="P290" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3025-oak-brushed-1744854</v>
@@ -15833,10 +15833,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N291" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-1744845.jpg</v>
       </c>
       <c r="O291" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-1744845.jpg</v>
       </c>
       <c r="P291" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3025-oak-1744845</v>
@@ -15886,10 +15886,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N292" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-1744844.jpg</v>
       </c>
       <c r="O292" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-1744844.jpg</v>
       </c>
       <c r="P292" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3025-oak-1744844</v>
@@ -15939,10 +15939,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N293" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-1744847.jpg</v>
       </c>
       <c r="O293" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-1744847.jpg</v>
       </c>
       <c r="P293" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3025-oak-1744847</v>
@@ -15992,10 +15992,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N294" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-1744848.jpg</v>
       </c>
       <c r="O294" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3025-oak-1744848.jpg</v>
       </c>
       <c r="P294" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3025-oak-1744848</v>
@@ -16045,10 +16045,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N295" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-4-oak-nougat-1739938.jpg</v>
       </c>
       <c r="O295" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-4-oak-nougat-1739938.jpg</v>
       </c>
       <c r="P295" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-trendtime-4-oak-nougat-1739938</v>
@@ -16098,10 +16098,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N296" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-4-oak-cream-1739937.jpg</v>
       </c>
       <c r="O296" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-4-oak-cream-1739937.jpg</v>
       </c>
       <c r="P296" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-trendtime-4-oak-cream-1739937</v>
@@ -16151,10 +16151,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N297" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-3-oak-nougat-1739933.jpg</v>
       </c>
       <c r="O297" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-3-oak-nougat-1739933.jpg</v>
       </c>
       <c r="P297" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-trendtime-3-oak-nougat-1739933</v>
@@ -16204,10 +16204,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N298" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-3-oak-1601582.jpg</v>
       </c>
       <c r="O298" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-3-oak-1601582.jpg</v>
       </c>
       <c r="P298" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-trendtime-3-oak-1601582</v>
@@ -16257,10 +16257,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N299" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-3-oak-cream-1739932.jpg</v>
       </c>
       <c r="O299" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-3-oak-cream-1739932.jpg</v>
       </c>
       <c r="P299" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-trendtime-3-oak-cream-1739932</v>
@@ -16310,10 +16310,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N300" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-walnut-1518117.jpg</v>
       </c>
       <c r="O300" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-walnut-1518117.jpg</v>
       </c>
       <c r="P300" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-walnut-1518117</v>
@@ -16363,10 +16363,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N301" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-walnut-1518118.jpg</v>
       </c>
       <c r="O301" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-walnut-1518118.jpg</v>
       </c>
       <c r="P301" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-walnut-1518118</v>
@@ -16416,10 +16416,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N302" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-larch-1739923.jpg</v>
       </c>
       <c r="O302" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-larch-1739923.jpg</v>
       </c>
       <c r="P302" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-larch-1739923</v>
@@ -16469,10 +16469,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N303" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-larch-smoked-soft-texture-1739904.jpg</v>
       </c>
       <c r="O303" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-larch-smoked-soft-texture-1739904.jpg</v>
       </c>
       <c r="P303" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-larch-smoked-soft-texture-1739904</v>
@@ -16522,10 +16522,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N304" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-ash-1270338.jpg</v>
       </c>
       <c r="O304" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-ash-1270338.jpg</v>
       </c>
       <c r="P304" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-ash-1270338</v>
@@ -16575,10 +16575,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N305" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1247127.jpg</v>
       </c>
       <c r="O305" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1247127.jpg</v>
       </c>
       <c r="P305" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-1247127</v>
@@ -16628,10 +16628,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N306" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1518125.jpg</v>
       </c>
       <c r="O306" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1518125.jpg</v>
       </c>
       <c r="P306" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-1518125</v>
@@ -16681,10 +16681,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N307" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1518128.jpg</v>
       </c>
       <c r="O307" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1518128.jpg</v>
       </c>
       <c r="P307" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-1518128</v>
@@ -16734,10 +16734,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N308" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-pure-1739912.jpg</v>
       </c>
       <c r="O308" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-pure-1739912.jpg</v>
       </c>
       <c r="P308" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-pure-1739912</v>
@@ -16787,10 +16787,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N309" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1739906.jpg</v>
       </c>
       <c r="O309" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1739906.jpg</v>
       </c>
       <c r="P309" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-1739906</v>
@@ -16840,10 +16840,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N310" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1739903.jpg</v>
       </c>
       <c r="O310" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1739903.jpg</v>
       </c>
       <c r="P310" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-1739903</v>
@@ -16893,10 +16893,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N311" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1739929.jpg</v>
       </c>
       <c r="O311" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1739929.jpg</v>
       </c>
       <c r="P311" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-1739929</v>
@@ -16946,10 +16946,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N312" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1518101.jpg</v>
       </c>
       <c r="O312" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1518101.jpg</v>
       </c>
       <c r="P312" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-1518101</v>
@@ -16999,10 +16999,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N313" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1247126.jpg</v>
       </c>
       <c r="O313" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1247126.jpg</v>
       </c>
       <c r="P313" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-1247126</v>
@@ -17052,10 +17052,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N314" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1358529.jpg</v>
       </c>
       <c r="O314" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1358529.jpg</v>
       </c>
       <c r="P314" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-1358529</v>
@@ -17105,10 +17105,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N315" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1518124.jpg</v>
       </c>
       <c r="O315" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1518124.jpg</v>
       </c>
       <c r="P315" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-1518124</v>
@@ -17158,10 +17158,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N316" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1518123.jpg</v>
       </c>
       <c r="O316" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-1518123.jpg</v>
       </c>
       <c r="P316" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-1518123</v>
@@ -17211,10 +17211,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N317" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-brushed-1739910.jpg</v>
       </c>
       <c r="O317" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-brushed-1739910.jpg</v>
       </c>
       <c r="P317" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-brushed-1739910</v>
@@ -17264,10 +17264,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N318" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-brushed-1739925.jpg</v>
       </c>
       <c r="O318" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-brushed-1739925.jpg</v>
       </c>
       <c r="P318" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-brushed-1739925</v>
@@ -17317,10 +17317,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N319" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-brushed-1368979.jpg</v>
       </c>
       <c r="O319" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-brushed-1368979.jpg</v>
       </c>
       <c r="P319" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-brushed-1368979</v>
@@ -17370,10 +17370,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N320" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-knotty-oak-1518102.jpg</v>
       </c>
       <c r="O320" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-knotty-oak-1518102.jpg</v>
       </c>
       <c r="P320" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-knotty-oak-1518102</v>
@@ -17423,10 +17423,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N321" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-beech-1518088.jpg</v>
       </c>
       <c r="O321" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-beech-1518088.jpg</v>
       </c>
       <c r="P321" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-beech-1518088</v>
@@ -17476,10 +17476,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N322" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-beech-1518103.jpg</v>
       </c>
       <c r="O322" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-beech-1518103.jpg</v>
       </c>
       <c r="P322" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-beech-1518103</v>
@@ -17529,10 +17529,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N323" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-european-maple-1518122.jpg</v>
       </c>
       <c r="O323" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-european-maple-1518122.jpg</v>
       </c>
       <c r="P323" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-european-maple-1518122</v>
@@ -17582,10 +17582,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N324" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-1366061.jpg</v>
       </c>
       <c r="O324" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-1366061.jpg</v>
       </c>
       <c r="P324" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-basic-11-5-oak-1366061</v>
@@ -17635,10 +17635,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N325" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-pure-1595165.jpg</v>
       </c>
       <c r="O325" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-pure-1595165.jpg</v>
       </c>
       <c r="P325" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-basic-11-5-oak-pure-1595165</v>
@@ -17688,10 +17688,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N326" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-1643835.jpg</v>
       </c>
       <c r="O326" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-1643835.jpg</v>
       </c>
       <c r="P326" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-basic-11-5-oak-1643835</v>
@@ -17741,10 +17741,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N327" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-1518249.jpg</v>
       </c>
       <c r="O327" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-1518249.jpg</v>
       </c>
       <c r="P327" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-basic-11-5-oak-1518249</v>
@@ -17794,10 +17794,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N328" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-1518262.jpg</v>
       </c>
       <c r="O328" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-1518262.jpg</v>
       </c>
       <c r="P328" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-basic-11-5-oak-1518262</v>
@@ -17847,10 +17847,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N329" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-1569685.jpg</v>
       </c>
       <c r="O329" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-1569685.jpg</v>
       </c>
       <c r="P329" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-basic-11-5-oak-1569685</v>
@@ -17900,10 +17900,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N330" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-1595131.jpg</v>
       </c>
       <c r="O330" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-1595131.jpg</v>
       </c>
       <c r="P330" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-basic-11-5-oak-1595131</v>
@@ -17953,10 +17953,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N331" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-1601464.jpg</v>
       </c>
       <c r="O331" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-1601464.jpg</v>
       </c>
       <c r="P331" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-basic-11-5-oak-1601464</v>
@@ -18006,10 +18006,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N332" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-1396114.jpg</v>
       </c>
       <c r="O332" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-1396114.jpg</v>
       </c>
       <c r="P332" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-basic-11-5-oak-1396114</v>
@@ -18059,10 +18059,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N333" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-brushed-1595135.jpg</v>
       </c>
       <c r="O333" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-brushed-1595135.jpg</v>
       </c>
       <c r="P333" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-basic-11-5-oak-brushed-1595135</v>
@@ -18112,10 +18112,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N334" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-brushed-1518264.jpg</v>
       </c>
       <c r="O334" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-oak-brushed-1518264.jpg</v>
       </c>
       <c r="P334" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-basic-11-5-oak-brushed-1518264</v>
@@ -18165,10 +18165,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N335" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-knotty-oak-1518245.jpg</v>
       </c>
       <c r="O335" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-knotty-oak-1518245.jpg</v>
       </c>
       <c r="P335" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-basic-11-5-knotty-oak-1518245</v>
@@ -18218,10 +18218,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N336" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-beech-1518246.jpg</v>
       </c>
       <c r="O336" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-beech-1518246.jpg</v>
       </c>
       <c r="P336" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-basic-11-5-beech-1518246</v>
@@ -18271,10 +18271,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N337" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-beech-1569684.jpg</v>
       </c>
       <c r="O337" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-basic-11-5-beech-1569684.jpg</v>
       </c>
       <c r="P337" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-basic-11-5-beech-1569684</v>
@@ -18324,10 +18324,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N338" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-soft-texture-1739902.jpg</v>
       </c>
       <c r="O338" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-classic-3060-oak-soft-texture-1739902.jpg</v>
       </c>
       <c r="P338" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-classic-3060-oak-soft-texture-1739902</v>
@@ -18377,10 +18377,10 @@
         <v>Engineered wood flooring: a real wood top layer on a multi-layer core for superior stability, with the warmth and character of natural timber.</v>
       </c>
       <c r="N339" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-3-oak-pure-1601580.jpg</v>
       </c>
       <c r="O339" t="str">
-        <v/>
+        <v>/images/products/oaken/engineered-flooring/parador-engineered-designer-trendtime-3-oak-pure-1601580.jpg</v>
       </c>
       <c r="P339" t="str">
         <v>/products/oaken/engineered-designer/engineered?product=engineered-designer-trendtime-3-oak-pure-1601580</v>
@@ -18589,10 +18589,10 @@
         <v>Solid wood flooring with high resistance to scratches, stains and fading, easy to install and maintain.</v>
       </c>
       <c r="N343" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/solid-wood/novawood-solid-wood-solid-parquet-thermowood-oak-solid-parquet.jpg</v>
       </c>
       <c r="O343" t="str">
-        <v/>
+        <v>/images/products/oaken/solid-wood/novawood-solid-wood-solid-parquet-thermowood-oak-solid-parquet.jpg</v>
       </c>
       <c r="P343" t="str">
         <v>/products/oaken/solid-wood?product=solid-wood-solid-parquet-thermowood-oak-solid-parquet</v>
@@ -18642,10 +18642,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N344" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-8-oak-loire-honey-1751649.jpg</v>
       </c>
       <c r="O344" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-8-oak-loire-honey-1751649.jpg</v>
       </c>
       <c r="P344" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-8-oak-loire-honey-1751649</v>
@@ -18695,10 +18695,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N345" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-8-oak-loire-beige-1751650.jpg</v>
       </c>
       <c r="O345" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-8-oak-loire-beige-1751650.jpg</v>
       </c>
       <c r="P345" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-8-oak-loire-beige-1751650</v>
@@ -18748,10 +18748,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N346" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-8-oak-loire-grey-1751651.jpg</v>
       </c>
       <c r="O346" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-8-oak-loire-grey-1751651.jpg</v>
       </c>
       <c r="P346" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-8-oak-loire-grey-1751651</v>
@@ -18801,10 +18801,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N347" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-5-malaga-1748676.jpg</v>
       </c>
       <c r="O347" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-5-malaga-1748676.jpg</v>
       </c>
       <c r="P347" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-5-malaga-1748676</v>
@@ -18854,10 +18854,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N348" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-8-oak-loire-grey-1748771.jpg</v>
       </c>
       <c r="O348" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-8-oak-loire-grey-1748771.jpg</v>
       </c>
       <c r="P348" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-8-oak-loire-grey-1748771</v>
@@ -18907,10 +18907,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N349" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-everglade-antique-1748792.jpg</v>
       </c>
       <c r="O349" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-everglade-antique-1748792.jpg</v>
       </c>
       <c r="P349" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-6-oak-everglade-antique-1748792</v>
@@ -18960,10 +18960,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N350" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-everglade-natural-1748791.jpg</v>
       </c>
       <c r="O350" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-everglade-natural-1748791.jpg</v>
       </c>
       <c r="P350" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-6-oak-everglade-natural-1748791</v>
@@ -19013,10 +19013,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N351" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-3-oak-mont-blanc-dark-brown-1748754.jpg</v>
       </c>
       <c r="O351" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-3-oak-mont-blanc-dark-brown-1748754.jpg</v>
       </c>
       <c r="P351" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-3-oak-mont-blanc-dark-brown-1748754</v>
@@ -19066,10 +19066,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N352" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-mont-blanc-brown-1748790.jpg</v>
       </c>
       <c r="O352" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-mont-blanc-brown-1748790.jpg</v>
       </c>
       <c r="P352" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-classic-1050-oak-mont-blanc-brown-1748790</v>
@@ -19119,10 +19119,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N353" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-3-oak-mont-blanc-sanded-1748753.jpg</v>
       </c>
       <c r="O353" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-3-oak-mont-blanc-sanded-1748753.jpg</v>
       </c>
       <c r="P353" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-3-oak-mont-blanc-sanded-1748753</v>
@@ -19172,10 +19172,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N354" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-3-larch-yukon-white-1748751.jpg</v>
       </c>
       <c r="O354" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-3-larch-yukon-white-1748751.jpg</v>
       </c>
       <c r="P354" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-3-larch-yukon-white-1748751</v>
@@ -19225,10 +19225,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N355" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-mont-blanc-natural-1748724.jpg</v>
       </c>
       <c r="O355" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-mont-blanc-natural-1748724.jpg</v>
       </c>
       <c r="P355" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-classic-1050-oak-mont-blanc-natural-1748724</v>
@@ -19278,10 +19278,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N356" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-mont-blanc-sanded-1748723.jpg</v>
       </c>
       <c r="O356" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-mont-blanc-sanded-1748723.jpg</v>
       </c>
       <c r="P356" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-classic-1050-oak-mont-blanc-sanded-1748723</v>
@@ -19331,10 +19331,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N357" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-larch-yukon-beige-1748722.jpg</v>
       </c>
       <c r="O357" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-larch-yukon-beige-1748722.jpg</v>
       </c>
       <c r="P357" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-classic-1050-larch-yukon-beige-1748722</v>
@@ -19384,10 +19384,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N358" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-larch-yukon-honey-1748721.jpg</v>
       </c>
       <c r="O358" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-larch-yukon-honey-1748721.jpg</v>
       </c>
       <c r="P358" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-classic-1050-larch-yukon-honey-1748721</v>
@@ -19437,10 +19437,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N359" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-rotterdam-1748720.jpg</v>
       </c>
       <c r="O359" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-rotterdam-1748720.jpg</v>
       </c>
       <c r="P359" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-classic-1050-rotterdam-1748720</v>
@@ -19490,10 +19490,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N360" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-1-shufflewood-harmony-1748705.jpg</v>
       </c>
       <c r="O360" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-1-shufflewood-harmony-1748705.jpg</v>
       </c>
       <c r="P360" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-1-shufflewood-harmony-1748705</v>
@@ -19543,10 +19543,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N361" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-crosscut-limed-1748383.jpg</v>
       </c>
       <c r="O361" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-crosscut-limed-1748383.jpg</v>
       </c>
       <c r="P361" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-400-oak-crosscut-limed-1748383</v>
@@ -19596,10 +19596,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N362" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-studioline-brown-grey-1748194.jpg</v>
       </c>
       <c r="O362" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-studioline-brown-grey-1748194.jpg</v>
       </c>
       <c r="P362" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-600-oak-studioline-brown-grey-1748194</v>
@@ -19649,10 +19649,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N363" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-montana-limed-1748193.jpg</v>
       </c>
       <c r="O363" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-montana-limed-1748193.jpg</v>
       </c>
       <c r="P363" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-600-oak-montana-limed-1748193</v>
@@ -19702,10 +19702,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N364" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-valere-pearl-grey-limed-1748192.jpg</v>
       </c>
       <c r="O364" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-valere-pearl-grey-limed-1748192.jpg</v>
       </c>
       <c r="P364" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-600-oak-valere-pearl-grey-limed-1748192</v>
@@ -19755,10 +19755,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N365" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-studioline-macchiato-1748186.jpg</v>
       </c>
       <c r="O365" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-studioline-macchiato-1748186.jpg</v>
       </c>
       <c r="P365" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-600-oak-studioline-macchiato-1748186</v>
@@ -19808,10 +19808,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N366" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-studioline-pure-1748187.jpg</v>
       </c>
       <c r="O366" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-studioline-pure-1748187.jpg</v>
       </c>
       <c r="P366" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-600-oak-studioline-pure-1748187</v>
@@ -19861,10 +19861,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N367" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-studioline-brown-1748185.jpg</v>
       </c>
       <c r="O367" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-studioline-brown-1748185.jpg</v>
       </c>
       <c r="P367" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-600-oak-studioline-brown-1748185</v>
@@ -19914,10 +19914,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N368" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-studioline-beige-1748183.jpg</v>
       </c>
       <c r="O368" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-studioline-beige-1748183.jpg</v>
       </c>
       <c r="P368" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-400-oak-studioline-beige-1748183</v>
@@ -19967,10 +19967,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N369" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-studioline-pearl-white-1748184.jpg</v>
       </c>
       <c r="O369" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-studioline-pearl-white-1748184.jpg</v>
       </c>
       <c r="P369" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-400-oak-studioline-pearl-white-1748184</v>
@@ -20020,10 +20020,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N370" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-hickory-1748182.jpg</v>
       </c>
       <c r="O370" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-hickory-1748182.jpg</v>
       </c>
       <c r="P370" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-400-hickory-1748182</v>
@@ -20073,10 +20073,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N371" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-natural-mix-crystal-white-1748180.jpg</v>
       </c>
       <c r="O371" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-natural-mix-crystal-white-1748180.jpg</v>
       </c>
       <c r="P371" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-400-oak-natural-mix-crystal-white-1748180</v>
@@ -20126,10 +20126,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N372" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-old-wood-beige-1748178.jpg</v>
       </c>
       <c r="O372" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-old-wood-beige-1748178.jpg</v>
       </c>
       <c r="P372" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-400-old-wood-beige-1748178</v>
@@ -20179,10 +20179,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N373" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-old-wood-white-1748179.jpg</v>
       </c>
       <c r="O373" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-old-wood-white-1748179.jpg</v>
       </c>
       <c r="P373" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-400-old-wood-white-1748179</v>
@@ -20232,10 +20232,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N374" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-natural-touch-1748177.jpg</v>
       </c>
       <c r="O374" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-natural-touch-1748177.jpg</v>
       </c>
       <c r="P374" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-400-natural-touch-1748177</v>
@@ -20285,10 +20285,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N375" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-caramel-1748176.jpg</v>
       </c>
       <c r="O375" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-caramel-1748176.jpg</v>
       </c>
       <c r="P375" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-400-oak-caramel-1748176</v>
@@ -20338,10 +20338,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N376" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-3-oak-skyline-white-1747862.jpg</v>
       </c>
       <c r="O376" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-3-oak-skyline-white-1747862.jpg</v>
       </c>
       <c r="P376" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-3-oak-skyline-white-1747862</v>
@@ -20391,10 +20391,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N377" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-3-oak-studioline-light-grey-1747865.jpg</v>
       </c>
       <c r="O377" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-3-oak-studioline-light-grey-1747865.jpg</v>
       </c>
       <c r="P377" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-3-oak-studioline-light-grey-1747865</v>
@@ -20444,10 +20444,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N378" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-3-oak-skyline-pearl-grey-1747861.jpg</v>
       </c>
       <c r="O378" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-3-oak-skyline-pearl-grey-1747861.jpg</v>
       </c>
       <c r="P378" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-3-oak-skyline-pearl-grey-1747861</v>
@@ -20497,10 +20497,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N379" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-nova-light-limed-1744353.jpg</v>
       </c>
       <c r="O379" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-nova-light-limed-1744353.jpg</v>
       </c>
       <c r="P379" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-600-oak-nova-light-limed-1744353</v>
@@ -20550,10 +20550,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N380" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-valere-pearl-grey-limed-1744355.jpg</v>
       </c>
       <c r="O380" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-valere-pearl-grey-limed-1744355.jpg</v>
       </c>
       <c r="P380" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-600-oak-valere-pearl-grey-limed-1744355</v>
@@ -20603,10 +20603,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N381" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-studioline-light-grey-1744696.jpg</v>
       </c>
       <c r="O381" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-studioline-light-grey-1744696.jpg</v>
       </c>
       <c r="P381" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-classic-1050-oak-studioline-light-grey-1744696</v>
@@ -20656,10 +20656,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N382" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-loft-pure-1744698.jpg</v>
       </c>
       <c r="O382" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-loft-pure-1744698.jpg</v>
       </c>
       <c r="P382" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-classic-1050-oak-loft-pure-1744698</v>
@@ -20709,10 +20709,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N383" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-loft-smoked-white-oiled-1744699.jpg</v>
       </c>
       <c r="O383" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-loft-smoked-white-oiled-1744699.jpg</v>
       </c>
       <c r="P383" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-classic-1050-oak-loft-smoked-white-oiled-1744699</v>
@@ -20762,10 +20762,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N384" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-studioline-light-grey-1744707.jpg</v>
       </c>
       <c r="O384" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-studioline-light-grey-1744707.jpg</v>
       </c>
       <c r="P384" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-6-oak-studioline-light-grey-1744707</v>
@@ -20815,10 +20815,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N385" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-loft-pure-1744709.jpg</v>
       </c>
       <c r="O385" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-loft-pure-1744709.jpg</v>
       </c>
       <c r="P385" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-6-oak-loft-pure-1744709</v>
@@ -20868,10 +20868,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N386" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-loft-smoked-white-oiled-1744710.jpg</v>
       </c>
       <c r="O386" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-loft-smoked-white-oiled-1744710.jpg</v>
       </c>
       <c r="P386" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-6-oak-loft-smoked-white-oiled-1744710</v>
@@ -20921,10 +20921,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N387" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-chronicle-1744348.jpg</v>
       </c>
       <c r="O387" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-chronicle-1744348.jpg</v>
       </c>
       <c r="P387" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-400-oak-chronicle-1744348</v>
@@ -20974,10 +20974,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N388" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-monterey-light-whitewashed-1744350.jpg</v>
       </c>
       <c r="O388" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-monterey-light-whitewashed-1744350.jpg</v>
       </c>
       <c r="P388" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-400-oak-monterey-light-whitewashed-1744350</v>
@@ -21027,10 +21027,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N389" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-nova-limed-1744352.jpg</v>
       </c>
       <c r="O389" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-nova-limed-1744352.jpg</v>
       </c>
       <c r="P389" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-600-oak-nova-limed-1744352</v>
@@ -21080,10 +21080,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N390" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-200-acacia-grey-1426414.jpg</v>
       </c>
       <c r="O390" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-200-acacia-grey-1426414.jpg</v>
       </c>
       <c r="P390" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-200-acacia-grey-1426414</v>
@@ -21133,10 +21133,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N391" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-200-oak-rough-sawn-white-1593573.jpg</v>
       </c>
       <c r="O391" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-200-oak-rough-sawn-white-1593573.jpg</v>
       </c>
       <c r="P391" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-200-oak-rough-sawn-white-1593573</v>
@@ -21186,10 +21186,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N392" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-200-californian-walnut-1426416.jpg</v>
       </c>
       <c r="O392" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-200-californian-walnut-1426416.jpg</v>
       </c>
       <c r="P392" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-200-californian-walnut-1426416</v>
@@ -21239,10 +21239,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N393" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-200-oak-sanded-1593997.jpg</v>
       </c>
       <c r="O393" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-200-oak-sanded-1593997.jpg</v>
       </c>
       <c r="P393" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-200-oak-sanded-1593997</v>
@@ -21292,10 +21292,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N394" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-200-oak-horizont-natural-1594001.jpg</v>
       </c>
       <c r="O394" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-200-oak-horizont-natural-1594001.jpg</v>
       </c>
       <c r="P394" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-200-oak-horizont-natural-1594001</v>
@@ -21345,10 +21345,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N395" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-200-oak-light-grey-1594000.jpg</v>
       </c>
       <c r="O395" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-200-oak-light-grey-1594000.jpg</v>
       </c>
       <c r="P395" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-200-oak-light-grey-1594000</v>
@@ -21398,10 +21398,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N396" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-ocean-teak-1426506.jpg</v>
       </c>
       <c r="O396" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-ocean-teak-1426506.jpg</v>
       </c>
       <c r="P396" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-400-ocean-teak-1426506</v>
@@ -21451,10 +21451,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N397" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-sanded-1426462.jpg</v>
       </c>
       <c r="O397" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-sanded-1426462.jpg</v>
       </c>
       <c r="P397" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-400-oak-sanded-1426462</v>
@@ -21504,10 +21504,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N398" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-horizont-natural-1593813.jpg</v>
       </c>
       <c r="O398" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-horizont-natural-1593813.jpg</v>
       </c>
       <c r="P398" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-400-oak-horizont-natural-1593813</v>
@@ -21557,10 +21557,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N399" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-natural-1593812.jpg</v>
       </c>
       <c r="O399" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-natural-1593812.jpg</v>
       </c>
       <c r="P399" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-400-oak-natural-1593812</v>
@@ -21610,10 +21610,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N400" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-sanded-1426542.jpg</v>
       </c>
       <c r="O400" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-sanded-1426542.jpg</v>
       </c>
       <c r="P400" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-400-oak-sanded-1426542</v>
@@ -21663,10 +21663,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N401" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-horizont-natural-1593797.jpg</v>
       </c>
       <c r="O401" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-horizont-natural-1593797.jpg</v>
       </c>
       <c r="P401" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-400-oak-horizont-natural-1593797</v>
@@ -21716,10 +21716,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N402" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-light-grey-1426530.jpg</v>
       </c>
       <c r="O402" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-light-grey-1426530.jpg</v>
       </c>
       <c r="P402" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-400-oak-light-grey-1426530</v>
@@ -21769,10 +21769,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N403" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-natural-grey-1593798.jpg</v>
       </c>
       <c r="O403" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-400-oak-natural-grey-1593798.jpg</v>
       </c>
       <c r="P403" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-400-oak-natural-grey-1593798</v>
@@ -21822,10 +21822,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N404" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-askada-white-limed-1593828.jpg</v>
       </c>
       <c r="O404" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-askada-white-limed-1593828.jpg</v>
       </c>
       <c r="P404" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-600-oak-askada-white-limed-1593828</v>
@@ -21875,10 +21875,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N405" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-avant-sanded-1593829.jpg</v>
       </c>
       <c r="O405" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-avant-sanded-1593829.jpg</v>
       </c>
       <c r="P405" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-600-oak-avant-sanded-1593829</v>
@@ -21928,10 +21928,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N406" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-horizont-natural-1593845.jpg</v>
       </c>
       <c r="O406" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-horizont-natural-1593845.jpg</v>
       </c>
       <c r="P406" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-600-oak-horizont-natural-1593845</v>
@@ -21981,10 +21981,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N407" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-montana-limed-1593830.jpg</v>
       </c>
       <c r="O407" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-basic-600-oak-montana-limed-1593830.jpg</v>
       </c>
       <c r="P407" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-basic-600-oak-montana-limed-1593830</v>
@@ -22034,10 +22034,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N408" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-smoked-1475603.jpg</v>
       </c>
       <c r="O408" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-smoked-1475603.jpg</v>
       </c>
       <c r="P408" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-classic-1050-oak-smoked-1475603</v>
@@ -22087,10 +22087,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N409" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-sanded-1475604.jpg</v>
       </c>
       <c r="O409" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-sanded-1475604.jpg</v>
       </c>
       <c r="P409" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-classic-1050-oak-sanded-1475604</v>
@@ -22140,10 +22140,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N410" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-monterey-light-whitewashed-1517684.jpg</v>
       </c>
       <c r="O410" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-monterey-light-whitewashed-1517684.jpg</v>
       </c>
       <c r="P410" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-classic-1050-oak-monterey-light-whitewashed-1517684</v>
@@ -22193,10 +22193,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N411" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-natural-mix-light-1730463.jpg</v>
       </c>
       <c r="O411" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-natural-mix-light-1730463.jpg</v>
       </c>
       <c r="P411" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-classic-1050-oak-natural-mix-light-1730463</v>
@@ -22246,10 +22246,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N412" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-prestige-natural-1601440.jpg</v>
       </c>
       <c r="O412" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-prestige-natural-1601440.jpg</v>
       </c>
       <c r="P412" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-classic-1050-oak-prestige-natural-1601440</v>
@@ -22299,10 +22299,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N413" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-skyline-pearl-grey-1601448.jpg</v>
       </c>
       <c r="O413" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-skyline-pearl-grey-1601448.jpg</v>
       </c>
       <c r="P413" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-classic-1050-oak-skyline-pearl-grey-1601448</v>
@@ -22352,10 +22352,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N414" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-skyline-white-1601447.jpg</v>
       </c>
       <c r="O414" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-skyline-white-1601447.jpg</v>
       </c>
       <c r="P414" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-classic-1050-oak-skyline-white-1601447</v>
@@ -22405,10 +22405,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N415" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-tradition-grey-beige-1517691.jpg</v>
       </c>
       <c r="O415" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-tradition-grey-beige-1517691.jpg</v>
       </c>
       <c r="P415" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-classic-1050-oak-tradition-grey-beige-1517691</v>
@@ -22458,10 +22458,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N416" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-tradition-natural-1601449.jpg</v>
       </c>
       <c r="O416" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-classic-1050-oak-tradition-natural-1601449.jpg</v>
       </c>
       <c r="P416" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-classic-1050-oak-tradition-natural-1601449</v>
@@ -22511,10 +22511,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N417" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-5-granite-anthracite-1743594.jpg</v>
       </c>
       <c r="O417" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-5-granite-anthracite-1743594.jpg</v>
       </c>
       <c r="P417" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-5-granite-anthracite-1743594</v>
@@ -22564,10 +22564,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N418" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-5-concrete-dark-grey-1743596.jpg</v>
       </c>
       <c r="O418" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-5-concrete-dark-grey-1743596.jpg</v>
       </c>
       <c r="P418" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-5-concrete-dark-grey-1743596</v>
@@ -22617,10 +22617,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N419" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-5-concrete-light-grey-1743595.jpg</v>
       </c>
       <c r="O419" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-5-concrete-light-grey-1743595.jpg</v>
       </c>
       <c r="P419" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-5-concrete-light-grey-1743595</v>
@@ -22670,10 +22670,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N420" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-5-granite-pearl-grey-1743593.jpg</v>
       </c>
       <c r="O420" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-5-granite-pearl-grey-1743593.jpg</v>
       </c>
       <c r="P420" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-5-granite-pearl-grey-1743593</v>
@@ -22723,10 +22723,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N421" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-5-crude-steel-1743600.jpg</v>
       </c>
       <c r="O421" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-5-crude-steel-1743600.jpg</v>
       </c>
       <c r="P421" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-5-crude-steel-1743600</v>
@@ -22776,10 +22776,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N422" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-nova-limed-1567468.jpg</v>
       </c>
       <c r="O422" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-nova-limed-1567468.jpg</v>
       </c>
       <c r="P422" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-6-oak-nova-limed-1567468</v>
@@ -22829,10 +22829,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N423" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-askada-white-limed-1567470.jpg</v>
       </c>
       <c r="O423" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-askada-white-limed-1567470.jpg</v>
       </c>
       <c r="P423" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-6-oak-askada-white-limed-1567470</v>
@@ -22882,10 +22882,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N424" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-avant-sanded-1567467.jpg</v>
       </c>
       <c r="O424" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-avant-sanded-1567467.jpg</v>
       </c>
       <c r="P424" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-6-oak-avant-sanded-1567467</v>
@@ -22935,10 +22935,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N425" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-castell-limed-1371173.jpg</v>
       </c>
       <c r="O425" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-castell-limed-1371173.jpg</v>
       </c>
       <c r="P425" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-6-oak-castell-limed-1371173</v>
@@ -22988,10 +22988,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N426" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-castell-smoked-1371174.jpg</v>
       </c>
       <c r="O426" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-castell-smoked-1371174.jpg</v>
       </c>
       <c r="P426" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-6-oak-castell-smoked-1371174</v>
@@ -23041,10 +23041,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N427" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-loft-grey-1730467.jpg</v>
       </c>
       <c r="O427" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-loft-grey-1730467.jpg</v>
       </c>
       <c r="P427" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-6-oak-loft-grey-1730467</v>
@@ -23094,10 +23094,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N428" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-loft-white-1730468.jpg</v>
       </c>
       <c r="O428" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-loft-white-1730468.jpg</v>
       </c>
       <c r="P428" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-6-oak-loft-white-1730468</v>
@@ -23147,10 +23147,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N429" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-mistral-grey-1567466.jpg</v>
       </c>
       <c r="O429" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-mistral-grey-1567466.jpg</v>
       </c>
       <c r="P429" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-6-oak-mistral-grey-1567466</v>
@@ -23200,10 +23200,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N430" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-montana-limed-1567473.jpg</v>
       </c>
       <c r="O430" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-montana-limed-1567473.jpg</v>
       </c>
       <c r="P430" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-6-oak-montana-limed-1567473</v>
@@ -23253,10 +23253,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N431" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-nova-light-limed-1567469.jpg</v>
       </c>
       <c r="O431" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-nova-light-limed-1567469.jpg</v>
       </c>
       <c r="P431" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-6-oak-nova-light-limed-1567469</v>
@@ -23306,10 +23306,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N432" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-skyline-pearl-grey-1601103.jpg</v>
       </c>
       <c r="O432" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-skyline-pearl-grey-1601103.jpg</v>
       </c>
       <c r="P432" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-6-oak-skyline-pearl-grey-1601103</v>
@@ -23359,10 +23359,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N433" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-valere-dark-limed-1567472.jpg</v>
       </c>
       <c r="O433" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-valere-dark-limed-1567472.jpg</v>
       </c>
       <c r="P433" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-6-oak-valere-dark-limed-1567472</v>
@@ -23412,10 +23412,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N434" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-valere-pearl-grey-limed-1567471.jpg</v>
       </c>
       <c r="O434" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-oak-valere-pearl-grey-limed-1567471.jpg</v>
       </c>
       <c r="P434" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-6-oak-valere-pearl-grey-limed-1567471</v>
@@ -23465,10 +23465,10 @@
         <v>Laminated and hybrid flooring that replicates the look of natural wood, with consistent texture and high resistance to scratches, stains and fading.</v>
       </c>
       <c r="N435" t="str">
-        <v>(none)</v>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-lumberjack-oak-1371172.jpg</v>
       </c>
       <c r="O435" t="str">
-        <v/>
+        <v>/images/products/oaken/laminated-flooring/parador-laminated-hybrid-trendtime-6-lumberjack-oak-1371172.jpg</v>
       </c>
       <c r="P435" t="str">
         <v>/products/oaken/laminated-hybrid/laminated?product=laminated-hybrid-trendtime-6-lumberjack-oak-1371172</v>
@@ -23518,10 +23518,10 @@
         <v>Outdoor decking in thermally modified and naturally durable hardwoods, built for terraces, pools and gardens.</v>
       </c>
       <c r="N436" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/deck-wood/lunawood-luna-deck-2-profix-2-26x92-profile.png</v>
       </c>
       <c r="O436" t="str">
-        <v/>
+        <v>/images/products/nordwood/deck-wood/lunawood-luna-deck-2-profix-2-26x92-profile.png</v>
       </c>
       <c r="P436" t="str">
         <v>/products/nordwood/deck-wood/real-wood?product=deck-wood-decking-hidden-profix-fixing-luna-deck-2-profix-2-26x92</v>
@@ -23571,10 +23571,10 @@
         <v>Outdoor decking in thermally modified and naturally durable hardwoods, built for terraces, pools and gardens.</v>
       </c>
       <c r="N437" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/deck-wood/lunawood-luna-deck-2-profix-2-26x117-profile.png</v>
       </c>
       <c r="O437" t="str">
-        <v/>
+        <v>/images/products/nordwood/deck-wood/lunawood-luna-deck-2-profix-2-26x117-profile.png</v>
       </c>
       <c r="P437" t="str">
         <v>/products/nordwood/deck-wood/real-wood?product=deck-wood-decking-hidden-profix-fixing-luna-deck-2-profix-2-26x117</v>
@@ -23624,10 +23624,10 @@
         <v>Outdoor decking in thermally modified and naturally durable hardwoods, built for terraces, pools and gardens.</v>
       </c>
       <c r="N438" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/deck-wood/lunawood-luna-shp-profix-2-26x117-profile.png</v>
       </c>
       <c r="O438" t="str">
-        <v/>
+        <v>/images/products/nordwood/deck-wood/lunawood-luna-shp-profix-2-26x117-profile.png</v>
       </c>
       <c r="P438" t="str">
         <v>/products/nordwood/deck-wood/real-wood?product=deck-wood-decking-hidden-profix-fixing-luna-shp-profix-2-26x117</v>
@@ -23677,10 +23677,10 @@
         <v>Outdoor decking in thermally modified and naturally durable hardwoods, built for terraces, pools and gardens.</v>
       </c>
       <c r="N439" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/deck-wood/lunawood-luna-shp-profix-2-26x140-profile.png</v>
       </c>
       <c r="O439" t="str">
-        <v/>
+        <v>/images/products/nordwood/deck-wood/lunawood-luna-shp-profix-2-26x140-profile.png</v>
       </c>
       <c r="P439" t="str">
         <v>/products/nordwood/deck-wood/real-wood?product=deck-wood-decking-hidden-profix-fixing-luna-shp-profix-2-26x140</v>
@@ -23730,10 +23730,10 @@
         <v>Outdoor decking in thermally modified and naturally durable hardwoods, built for terraces, pools and gardens.</v>
       </c>
       <c r="N440" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/deck-wood/lunawood-luna-shp-profix-2-26x140-brushed-profile.png</v>
       </c>
       <c r="O440" t="str">
-        <v/>
+        <v>/images/products/nordwood/deck-wood/lunawood-luna-shp-profix-2-26x140-brushed-profile.png</v>
       </c>
       <c r="P440" t="str">
         <v>/products/nordwood/deck-wood/real-wood?product=deck-wood-decking-hidden-profix-fixing-luna-shp-profix-2-26x140-brushed</v>
@@ -23783,10 +23783,10 @@
         <v>Outdoor decking in thermally modified and naturally durable hardwoods, built for terraces, pools and gardens.</v>
       </c>
       <c r="N441" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/deck-wood/lunawood-luna-shp-profix-3-32x166-brushed-profile.png</v>
       </c>
       <c r="O441" t="str">
-        <v/>
+        <v>/images/products/nordwood/deck-wood/lunawood-luna-shp-profix-3-32x166-brushed-profile.png</v>
       </c>
       <c r="P441" t="str">
         <v>/products/nordwood/deck-wood/real-wood?product=deck-wood-decking-hidden-profix-fixing-luna-shp-profix-3-32x166-brushed</v>
@@ -23836,10 +23836,10 @@
         <v>Outdoor decking in thermally modified and naturally durable hardwoods, built for terraces, pools and gardens.</v>
       </c>
       <c r="N442" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/deck-wood/lunawood-luna-shp-profix-3-40x185-profile.png</v>
       </c>
       <c r="O442" t="str">
-        <v/>
+        <v>/images/products/nordwood/deck-wood/lunawood-luna-shp-profix-3-40x185-profile.png</v>
       </c>
       <c r="P442" t="str">
         <v>/products/nordwood/deck-wood/real-wood?product=deck-wood-decking-hidden-profix-fixing-luna-shp-profix-3-40x185</v>
@@ -24048,10 +24048,10 @@
         <v>Outdoor decking in thermally modified and naturally durable hardwoods, built for terraces, pools and gardens.</v>
       </c>
       <c r="N446" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/deck-wood/novawood-deck-wood-decking-nova-kd-iroko-decking.jpg</v>
       </c>
       <c r="O446" t="str">
-        <v/>
+        <v>/images/products/nordwood/deck-wood/novawood-deck-wood-decking-nova-kd-iroko-decking.jpg</v>
       </c>
       <c r="P446" t="str">
         <v>/products/nordwood/deck-wood/real-wood?product=deck-wood-decking-nova-kd-iroko-decking</v>
@@ -24101,10 +24101,10 @@
         <v>Outdoor decking in thermally modified and naturally durable hardwoods, built for terraces, pools and gardens.</v>
       </c>
       <c r="N447" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/deck-wood/novawood-deck-wood-decking-nova-teak-decking.jpg</v>
       </c>
       <c r="O447" t="str">
-        <v/>
+        <v>/images/products/nordwood/deck-wood/novawood-deck-wood-decking-nova-teak-decking.jpg</v>
       </c>
       <c r="P447" t="str">
         <v>/products/nordwood/deck-wood/real-wood?product=deck-wood-decking-nova-teak-decking</v>
@@ -24366,10 +24366,10 @@
         <v>Wood cladding and wall panels that combine visual appeal with durability and structural integrity.</v>
       </c>
       <c r="N452" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-triple-32x140-profile.png</v>
       </c>
       <c r="O452" t="str">
-        <v/>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-triple-32x140-profile.png</v>
       </c>
       <c r="P452" t="str">
         <v>/products/nordwood/wall-cladding?product=wall-cladding-3d-claddings-luna-triple-32x140</v>
@@ -24419,10 +24419,10 @@
         <v>Wood cladding and wall panels that combine visual appeal with durability and structural integrity.</v>
       </c>
       <c r="N453" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-duple-32x140-profile.png</v>
       </c>
       <c r="O453" t="str">
-        <v/>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-duple-32x140-profile.png</v>
       </c>
       <c r="P453" t="str">
         <v>/products/nordwood/wall-cladding?product=wall-cladding-3d-claddings-luna-duple-32x140</v>
@@ -24472,10 +24472,10 @@
         <v>Wood cladding and wall panels that combine visual appeal with durability and structural integrity.</v>
       </c>
       <c r="N454" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-duo-32x140-profile.png</v>
       </c>
       <c r="O454" t="str">
-        <v/>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-duo-32x140-profile.png</v>
       </c>
       <c r="P454" t="str">
         <v>/products/nordwood/wall-cladding?product=wall-cladding-3d-claddings-luna-duo-32x140</v>
@@ -24525,10 +24525,10 @@
         <v>Wood cladding and wall panels that combine visual appeal with durability and structural integrity.</v>
       </c>
       <c r="N455" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-block-32x140-profile.png</v>
       </c>
       <c r="O455" t="str">
-        <v/>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-block-32x140-profile.png</v>
       </c>
       <c r="P455" t="str">
         <v>/products/nordwood/wall-cladding?product=wall-cladding-3d-claddings-luna-block-32x140</v>
@@ -24578,10 +24578,10 @@
         <v>Wood cladding and wall panels that combine visual appeal with durability and structural integrity.</v>
       </c>
       <c r="N456" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-trio-26x92-profile.png</v>
       </c>
       <c r="O456" t="str">
-        <v/>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-trio-26x92-profile.png</v>
       </c>
       <c r="P456" t="str">
         <v>/products/nordwood/wall-cladding?product=wall-cladding-3d-claddings-luna-trio-26x92</v>
@@ -24631,10 +24631,10 @@
         <v>Wood cladding and wall panels that combine visual appeal with durability and structural integrity.</v>
       </c>
       <c r="N457" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-femma-26x142-profile.png</v>
       </c>
       <c r="O457" t="str">
-        <v/>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-femma-26x142-profile.png</v>
       </c>
       <c r="P457" t="str">
         <v>/products/nordwood/wall-cladding?product=wall-cladding-3d-claddings-luna-femma-26x142</v>
@@ -24684,10 +24684,10 @@
         <v>Wood cladding and wall panels that combine visual appeal with durability and structural integrity.</v>
       </c>
       <c r="N458" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-dual-26x142-profile.png</v>
       </c>
       <c r="O458" t="str">
-        <v/>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-dual-26x142-profile.png</v>
       </c>
       <c r="P458" t="str">
         <v>/products/nordwood/wall-cladding?product=wall-cladding-3d-claddings-luna-dual-26x142</v>
@@ -24737,10 +24737,10 @@
         <v>Wood cladding and wall panels that combine visual appeal with durability and structural integrity.</v>
       </c>
       <c r="N459" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-aalto-32x142-profile.png</v>
       </c>
       <c r="O459" t="str">
-        <v/>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-aalto-32x142-profile.png</v>
       </c>
       <c r="P459" t="str">
         <v>/products/nordwood/wall-cladding?product=wall-cladding-3d-claddings-luna-aalto-32x142</v>
@@ -24790,10 +24790,10 @@
         <v>Wood cladding and wall panels that combine visual appeal with durability and structural integrity.</v>
       </c>
       <c r="N460" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-panel-system-19x68-profile.png</v>
       </c>
       <c r="O460" t="str">
-        <v/>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-panel-system-19x68-profile.png</v>
       </c>
       <c r="P460" t="str">
         <v>/products/nordwood/wall-cladding?product=wall-cladding-luna-panel-system-interior-luna-panel-system-19x68</v>
@@ -24843,10 +24843,10 @@
         <v>Wood cladding and wall panels that combine visual appeal with durability and structural integrity.</v>
       </c>
       <c r="N461" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-panel-system-19x117-profile.png</v>
       </c>
       <c r="O461" t="str">
-        <v/>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-panel-system-19x117-profile.png</v>
       </c>
       <c r="P461" t="str">
         <v>/products/nordwood/wall-cladding?product=wall-cladding-luna-panel-system-interior-luna-panel-system-19x117-end-matched</v>
@@ -24896,10 +24896,10 @@
         <v>Wood cladding and wall panels that combine visual appeal with durability and structural integrity.</v>
       </c>
       <c r="N462" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-panel-system-19x140-profile.png</v>
       </c>
       <c r="O462" t="str">
-        <v/>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-panel-system-19x140-profile.png</v>
       </c>
       <c r="P462" t="str">
         <v>/products/nordwood/wall-cladding?product=wall-cladding-luna-panel-system-interior-luna-panel-system-19x140-end-matched</v>
@@ -24949,10 +24949,10 @@
         <v>Wood cladding and wall panels that combine visual appeal with durability and structural integrity.</v>
       </c>
       <c r="N463" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-panel-system-26x92-profile.png</v>
       </c>
       <c r="O463" t="str">
-        <v/>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-panel-system-26x92-profile.png</v>
       </c>
       <c r="P463" t="str">
         <v>/products/nordwood/wall-cladding?product=wall-cladding-luna-panel-system-interior-luna-panel-system-26x92</v>
@@ -25002,10 +25002,10 @@
         <v>Wood cladding and wall panels that combine visual appeal with durability and structural integrity.</v>
       </c>
       <c r="N464" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-panel-system-42x68-profile.png</v>
       </c>
       <c r="O464" t="str">
-        <v/>
+        <v>/images/products/nordwood/wall-cladding/lunawood-luna-panel-system-42x68-profile.png</v>
       </c>
       <c r="P464" t="str">
         <v>/products/nordwood/wall-cladding?product=wall-cladding-luna-panel-system-interior-luna-panel-system-42x68</v>
@@ -25320,10 +25320,10 @@
         <v>Wood cladding and wall panels that combine visual appeal with durability and structural integrity.</v>
       </c>
       <c r="N470" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/wall-cladding/novawood-wall-cladding-cladding-nova-radiata-pine-cladding.jpg</v>
       </c>
       <c r="O470" t="str">
-        <v/>
+        <v>/images/products/nordwood/wall-cladding/novawood-wall-cladding-cladding-nova-radiata-pine-cladding.jpg</v>
       </c>
       <c r="P470" t="str">
         <v>/products/nordwood/wall-cladding?product=wall-cladding-cladding-nova-radiata-pine-cladding</v>
@@ -25373,10 +25373,10 @@
         <v>Wood cladding and wall panels that combine visual appeal with durability and structural integrity.</v>
       </c>
       <c r="N471" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/wall-cladding/novawood-wall-cladding-cladding-nova-kd-iroko-cladding.jpg</v>
       </c>
       <c r="O471" t="str">
-        <v/>
+        <v>/images/products/nordwood/wall-cladding/novawood-wall-cladding-cladding-nova-kd-iroko-cladding.jpg</v>
       </c>
       <c r="P471" t="str">
         <v>/products/nordwood/wall-cladding?product=wall-cladding-cladding-nova-kd-iroko-cladding</v>
@@ -25426,10 +25426,10 @@
         <v>Wood cladding and wall panels that combine visual appeal with durability and structural integrity.</v>
       </c>
       <c r="N472" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/wall-cladding/novawood-wall-cladding-interior-wall-panels-interior-wall-panels.jpg</v>
       </c>
       <c r="O472" t="str">
-        <v/>
+        <v>/images/products/nordwood/wall-cladding/novawood-wall-cladding-interior-wall-panels-interior-wall-panels.jpg</v>
       </c>
       <c r="P472" t="str">
         <v>/products/nordwood/wall-cladding?product=wall-cladding-interior-wall-panels-interior-wall-panels</v>
@@ -25479,10 +25479,10 @@
         <v>Wood ceiling panels and linings for refined ceilings with easy installation.</v>
       </c>
       <c r="N473" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/ceiling-sofit/lunawood-luna-panel-system-19x68-profile.png</v>
       </c>
       <c r="O473" t="str">
-        <v/>
+        <v>/images/products/nordwood/ceiling-sofit/lunawood-luna-panel-system-19x68-profile.png</v>
       </c>
       <c r="P473" t="str">
         <v>/products/nordwood/ceiling?product=ceiling-luna-panel-system-interior-luna-panel-system-19x68</v>
@@ -25532,10 +25532,10 @@
         <v>Wood ceiling panels and linings for refined ceilings with easy installation.</v>
       </c>
       <c r="N474" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/ceiling-sofit/lunawood-luna-panel-system-19x117-profile.png</v>
       </c>
       <c r="O474" t="str">
-        <v/>
+        <v>/images/products/nordwood/ceiling-sofit/lunawood-luna-panel-system-19x117-profile.png</v>
       </c>
       <c r="P474" t="str">
         <v>/products/nordwood/ceiling?product=ceiling-luna-panel-system-interior-luna-panel-system-19x117-end-matched</v>
@@ -25585,10 +25585,10 @@
         <v>Wood ceiling panels and linings for refined ceilings with easy installation.</v>
       </c>
       <c r="N475" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/ceiling-sofit/lunawood-luna-panel-system-19x140-profile.png</v>
       </c>
       <c r="O475" t="str">
-        <v/>
+        <v>/images/products/nordwood/ceiling-sofit/lunawood-luna-panel-system-19x140-profile.png</v>
       </c>
       <c r="P475" t="str">
         <v>/products/nordwood/ceiling?product=ceiling-luna-panel-system-interior-luna-panel-system-19x140-end-matched</v>
@@ -25638,10 +25638,10 @@
         <v>Wood ceiling panels and linings for refined ceilings with easy installation.</v>
       </c>
       <c r="N476" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/ceiling-sofit/lunawood-luna-panel-system-26x92-profile.png</v>
       </c>
       <c r="O476" t="str">
-        <v/>
+        <v>/images/products/nordwood/ceiling-sofit/lunawood-luna-panel-system-26x92-profile.png</v>
       </c>
       <c r="P476" t="str">
         <v>/products/nordwood/ceiling?product=ceiling-luna-panel-system-interior-luna-panel-system-26x92</v>
@@ -25691,10 +25691,10 @@
         <v>Wood ceiling panels and linings for refined ceilings with easy installation.</v>
       </c>
       <c r="N477" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/ceiling-sofit/lunawood-luna-panel-system-42x68-profile.png</v>
       </c>
       <c r="O477" t="str">
-        <v/>
+        <v>/images/products/nordwood/ceiling-sofit/lunawood-luna-panel-system-42x68-profile.png</v>
       </c>
       <c r="P477" t="str">
         <v>/products/nordwood/ceiling?product=ceiling-luna-panel-system-interior-luna-panel-system-42x68</v>
@@ -25744,10 +25744,10 @@
         <v>Wood ceiling panels and linings for refined ceilings with easy installation.</v>
       </c>
       <c r="N478" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/ceiling-sofit/lunawood-luna-edge-15x92-profile.png</v>
       </c>
       <c r="O478" t="str">
-        <v/>
+        <v>/images/products/nordwood/ceiling-sofit/lunawood-luna-edge-15x92-profile.png</v>
       </c>
       <c r="P478" t="str">
         <v>/products/nordwood/ceiling?product=ceiling-interior-sauna-products-luna-edge-15x92</v>
@@ -25797,10 +25797,10 @@
         <v>Wood ceiling panels and linings for refined ceilings with easy installation.</v>
       </c>
       <c r="N479" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/ceiling-sofit/lunawood-luna-edge-15x117-profile.png</v>
       </c>
       <c r="O479" t="str">
-        <v/>
+        <v>/images/products/nordwood/ceiling-sofit/lunawood-luna-edge-15x117-profile.png</v>
       </c>
       <c r="P479" t="str">
         <v>/products/nordwood/ceiling?product=ceiling-interior-sauna-products-luna-edge-15x117</v>
@@ -25850,10 +25850,10 @@
         <v>Wood ceiling panels and linings for refined ceilings with easy installation.</v>
       </c>
       <c r="N480" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/ceiling-sofit/lunawood-luna-round-15x92-profile.png</v>
       </c>
       <c r="O480" t="str">
-        <v/>
+        <v>/images/products/nordwood/ceiling-sofit/lunawood-luna-round-15x92-profile.png</v>
       </c>
       <c r="P480" t="str">
         <v>/products/nordwood/ceiling?product=ceiling-interior-sauna-products-luna-round-15x92</v>
@@ -25903,10 +25903,10 @@
         <v>Wood ceiling panels and linings for refined ceilings with easy installation.</v>
       </c>
       <c r="N481" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/ceiling-sofit/lunawood-luna-shp-26x92-sauna-profile.png</v>
       </c>
       <c r="O481" t="str">
-        <v/>
+        <v>/images/products/nordwood/ceiling-sofit/lunawood-luna-shp-26x92-sauna-profile.png</v>
       </c>
       <c r="P481" t="str">
         <v>/products/nordwood/ceiling?product=ceiling-interior-sauna-products-luna-shp-26x92-sauna</v>
@@ -25956,10 +25956,10 @@
         <v>Wood ceiling panels and linings for refined ceilings with easy installation.</v>
       </c>
       <c r="N482" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/wall-cladding/novawood-wall-cladding-interior-wall-panels-interior-wall-panels.jpg</v>
       </c>
       <c r="O482" t="str">
-        <v/>
+        <v>/images/products/nordwood/wall-cladding/novawood-wall-cladding-interior-wall-panels-interior-wall-panels.jpg</v>
       </c>
       <c r="P482" t="str">
         <v>/products/nordwood/ceiling?product=ceiling-interior-wall-panels-interior-wall-panels</v>
@@ -26009,10 +26009,10 @@
         <v>Wood ceiling panels and linings for refined ceilings with easy installation.</v>
       </c>
       <c r="N483" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/ceiling-sofit/novawood-ceiling-solid-panel-solid-panel.jpg</v>
       </c>
       <c r="O483" t="str">
-        <v/>
+        <v>/images/products/nordwood/ceiling-sofit/novawood-ceiling-solid-panel-solid-panel.jpg</v>
       </c>
       <c r="P483" t="str">
         <v>/products/nordwood/ceiling?product=ceiling-solid-panel-solid-panel</v>
@@ -26115,10 +26115,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N485" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-uts-19x117-profile.png</v>
       </c>
       <c r="O485" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-uts-19x117-profile.png</v>
       </c>
       <c r="P485" t="str">
         <v>/products/nordwood/facade?product=facade-claddings-t-g-luna-uts-19x117</v>
@@ -26168,10 +26168,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N486" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-utv-19x117-profile.png</v>
       </c>
       <c r="O486" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-utv-19x117-profile.png</v>
       </c>
       <c r="P486" t="str">
         <v>/products/nordwood/facade?product=facade-claddings-t-g-luna-utv-19x117</v>
@@ -26221,10 +26221,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N487" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-utv-19x140-profile.png</v>
       </c>
       <c r="O487" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-utv-19x140-profile.png</v>
       </c>
       <c r="P487" t="str">
         <v>/products/nordwood/facade?product=facade-claddings-t-g-luna-utv-19x140</v>
@@ -26274,10 +26274,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N488" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-tgv-19x140-profile.png</v>
       </c>
       <c r="O488" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-tgv-19x140-profile.png</v>
       </c>
       <c r="P488" t="str">
         <v>/products/nordwood/facade?product=facade-claddings-t-g-luna-tgv-19x140</v>
@@ -26327,10 +26327,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N489" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-uyls-20x140-profile.png</v>
       </c>
       <c r="O489" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-uyls-20x140-profile.png</v>
       </c>
       <c r="P489" t="str">
         <v>/products/nordwood/facade?product=facade-claddings-t-g-luna-uyls-20x140</v>
@@ -26380,10 +26380,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N490" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-layer-19x142-brushed-profile.png</v>
       </c>
       <c r="O490" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-layer-19x142-brushed-profile.png</v>
       </c>
       <c r="P490" t="str">
         <v>/products/nordwood/facade?product=facade-claddings-t-g-luna-layer-19x142-brushed</v>
@@ -26433,10 +26433,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N491" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-layer-19x188-brushed-profile.png</v>
       </c>
       <c r="O491" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-layer-19x188-brushed-profile.png</v>
       </c>
       <c r="P491" t="str">
         <v>/products/nordwood/facade?product=facade-claddings-t-g-luna-layer-19x188-brushed</v>
@@ -26486,10 +26486,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N492" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-pure-hf-20x142-profile.png</v>
       </c>
       <c r="O492" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-pure-hf-20x142-profile.png</v>
       </c>
       <c r="P492" t="str">
         <v>/products/nordwood/facade?product=facade-hidden-fixing-cladding-luna-pure-hf-20x142</v>
@@ -26539,10 +26539,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N493" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-bevel-hf-26x142-profile.png</v>
       </c>
       <c r="O493" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-bevel-hf-26x142-profile.png</v>
       </c>
       <c r="P493" t="str">
         <v>/products/nordwood/facade?product=facade-hidden-fixing-cladding-luna-bevel-hf-26x142</v>
@@ -26592,10 +26592,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N494" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-sharp-hf-20x142-profile.png</v>
       </c>
       <c r="O494" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-sharp-hf-20x142-profile.png</v>
       </c>
       <c r="P494" t="str">
         <v>/products/nordwood/facade?product=facade-hidden-fixing-cladding-luna-sharp-hf-20x142</v>
@@ -26645,10 +26645,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N495" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-sharp-hf-20x142-brushed-profile.png</v>
       </c>
       <c r="O495" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-sharp-hf-20x142-brushed-profile.png</v>
       </c>
       <c r="P495" t="str">
         <v>/products/nordwood/facade?product=facade-hidden-fixing-cladding-luna-sharp-hf-20x142-brushed</v>
@@ -26698,10 +26698,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N496" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-classic-hf-21x117-brushed-profile.png</v>
       </c>
       <c r="O496" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-classic-hf-21x117-brushed-profile.png</v>
       </c>
       <c r="P496" t="str">
         <v>/products/nordwood/facade?product=facade-hidden-fixing-cladding-luna-classic-hf-21x117-brushed</v>
@@ -26751,10 +26751,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N497" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-classic-line-hf-21x117-brushed-profile.png</v>
       </c>
       <c r="O497" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-classic-line-hf-21x117-brushed-profile.png</v>
       </c>
       <c r="P497" t="str">
         <v>/products/nordwood/facade?product=facade-hidden-fixing-cladding-luna-classic-line-hf-21x117-brushed</v>
@@ -26804,10 +26804,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N498" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-grain-hf-19x142-brushed-profile.png</v>
       </c>
       <c r="O498" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-grain-hf-19x142-brushed-profile.png</v>
       </c>
       <c r="P498" t="str">
         <v>/products/nordwood/facade?product=facade-hidden-fixing-cladding-luna-grain-hf-19x142-brushed</v>
@@ -26857,10 +26857,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N499" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-triple-hf-26x140-profile.png</v>
       </c>
       <c r="O499" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-triple-hf-26x140-profile.png</v>
       </c>
       <c r="P499" t="str">
         <v>/products/nordwood/facade?product=facade-hidden-fixing-cladding-luna-triple-hf-26x140</v>
@@ -26910,10 +26910,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N500" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-19x92-profile.png</v>
       </c>
       <c r="O500" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-19x92-profile.png</v>
       </c>
       <c r="P500" t="str">
         <v>/products/nordwood/facade?product=facade-battens-luna-shp-19x92</v>
@@ -26963,10 +26963,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N501" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-19x117-profile.png</v>
       </c>
       <c r="O501" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-19x117-profile.png</v>
       </c>
       <c r="P501" t="str">
         <v>/products/nordwood/facade?product=facade-battens-luna-shp-19x117</v>
@@ -27016,10 +27016,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N502" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-19x140-profile.png</v>
       </c>
       <c r="O502" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-19x140-profile.png</v>
       </c>
       <c r="P502" t="str">
         <v>/products/nordwood/facade?product=facade-battens-luna-shp-19x140</v>
@@ -27069,10 +27069,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N503" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-26x92-profile.png</v>
       </c>
       <c r="O503" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-26x92-profile.png</v>
       </c>
       <c r="P503" t="str">
         <v>/products/nordwood/facade?product=facade-battens-luna-shp-26x92</v>
@@ -27122,10 +27122,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N504" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-26x117-profile.png</v>
       </c>
       <c r="O504" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-26x117-profile.png</v>
       </c>
       <c r="P504" t="str">
         <v>/products/nordwood/facade?product=facade-battens-luna-shp-26x117</v>
@@ -27175,10 +27175,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N505" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-26x140-profile.png</v>
       </c>
       <c r="O505" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-26x140-profile.png</v>
       </c>
       <c r="P505" t="str">
         <v>/products/nordwood/facade?product=facade-battens-luna-shp-26x140</v>
@@ -27228,10 +27228,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N506" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-40x185-profile.png</v>
       </c>
       <c r="O506" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-40x185-profile.png</v>
       </c>
       <c r="P506" t="str">
         <v>/products/nordwood/facade?product=facade-battens-luna-shp-40x185</v>
@@ -27281,10 +27281,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N507" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-42x42-profile.png</v>
       </c>
       <c r="O507" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-42x42-profile.png</v>
       </c>
       <c r="P507" t="str">
         <v>/products/nordwood/facade?product=facade-battens-luna-shp-42x42</v>
@@ -27334,10 +27334,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N508" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-42x68-profile.png</v>
       </c>
       <c r="O508" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-42x68-profile.png</v>
       </c>
       <c r="P508" t="str">
         <v>/products/nordwood/facade?product=facade-battens-luna-shp-42x68</v>
@@ -27387,10 +27387,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N509" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-42x92-profile.png</v>
       </c>
       <c r="O509" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-42x92-profile.png</v>
       </c>
       <c r="P509" t="str">
         <v>/products/nordwood/facade?product=facade-battens-luna-shp-42x92</v>
@@ -27440,10 +27440,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N510" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-42x117-profile.png</v>
       </c>
       <c r="O510" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-42x117-profile.png</v>
       </c>
       <c r="P510" t="str">
         <v>/products/nordwood/facade?product=facade-battens-luna-shp-42x117</v>
@@ -27493,10 +27493,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N511" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-42x140-profile.png</v>
       </c>
       <c r="O511" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-shp-42x140-profile.png</v>
       </c>
       <c r="P511" t="str">
         <v>/products/nordwood/facade?product=facade-battens-luna-shp-42x140</v>
@@ -27546,10 +27546,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N512" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-parallelogram-sss-20x92-profile.png</v>
       </c>
       <c r="O512" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-parallelogram-sss-20x92-profile.png</v>
       </c>
       <c r="P512" t="str">
         <v>/products/nordwood/facade?product=facade-battens-luna-parallelogram-sss-20x92</v>
@@ -27599,10 +27599,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N513" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-parallelogram-sss-26x68-profile.png</v>
       </c>
       <c r="O513" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-parallelogram-sss-26x68-profile.png</v>
       </c>
       <c r="P513" t="str">
         <v>/products/nordwood/facade?product=facade-battens-luna-parallelogram-sss-26x68</v>
@@ -27652,10 +27652,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N514" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-half-parallelogram-hss-28-42x42-profile.png</v>
       </c>
       <c r="O514" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-half-parallelogram-hss-28-42x42-profile.png</v>
       </c>
       <c r="P514" t="str">
         <v>/products/nordwood/facade?product=facade-battens-luna-half-parallelogram-hss-28-42x42</v>
@@ -27705,10 +27705,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N515" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-arctic-layer-19x142-brushed-profile.png</v>
       </c>
       <c r="O515" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-arctic-layer-19x142-brushed-profile.png</v>
       </c>
       <c r="P515" t="str">
         <v>/products/nordwood/facade?product=facade-luna-arctic-silver-grey-finish-luna-arctic-layer-19x142-brushed</v>
@@ -27758,10 +27758,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N516" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-arctic-layer-19x188-brushed-profile.png</v>
       </c>
       <c r="O516" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-arctic-layer-19x188-brushed-profile.png</v>
       </c>
       <c r="P516" t="str">
         <v>/products/nordwood/facade?product=facade-luna-arctic-silver-grey-finish-luna-arctic-layer-19x188-brushed</v>
@@ -27811,10 +27811,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N517" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-arctic-shp-19x92-brushed-profile.png</v>
       </c>
       <c r="O517" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-arctic-shp-19x92-brushed-profile.png</v>
       </c>
       <c r="P517" t="str">
         <v>/products/nordwood/facade?product=facade-luna-arctic-silver-grey-finish-luna-arctic-shp-19x92-brushed</v>
@@ -27864,10 +27864,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N518" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-arctic-shp-19x117-brushed-profile.png</v>
       </c>
       <c r="O518" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-arctic-shp-19x117-brushed-profile.png</v>
       </c>
       <c r="P518" t="str">
         <v>/products/nordwood/facade?product=facade-luna-arctic-silver-grey-finish-luna-arctic-shp-19x117-brushed</v>
@@ -27917,10 +27917,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N519" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-arctic-triple-32x140-brushed-profile.png</v>
       </c>
       <c r="O519" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-arctic-triple-32x140-brushed-profile.png</v>
       </c>
       <c r="P519" t="str">
         <v>/products/nordwood/facade?product=facade-luna-arctic-silver-grey-finish-luna-arctic-triple-32x140-brushed</v>
@@ -27970,10 +27970,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N520" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/facade/lunawood-luna-arctic-sharp-hf-20x142-brushed-profile.png</v>
       </c>
       <c r="O520" t="str">
-        <v/>
+        <v>/images/products/nordwood/facade/lunawood-luna-arctic-sharp-hf-20x142-brushed-profile.png</v>
       </c>
       <c r="P520" t="str">
         <v>/products/nordwood/facade?product=facade-luna-arctic-silver-grey-finish-luna-arctic-sharp-hf-20x142-brushed</v>
@@ -28288,10 +28288,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N526" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/wall-cladding/novawood-wall-cladding-cladding-nova-radiata-pine-cladding.jpg</v>
       </c>
       <c r="O526" t="str">
-        <v/>
+        <v>/images/products/nordwood/wall-cladding/novawood-wall-cladding-cladding-nova-radiata-pine-cladding.jpg</v>
       </c>
       <c r="P526" t="str">
         <v>/products/nordwood/facade?product=facade-facade-cladding-nova-radiata-pine-cladding</v>
@@ -28341,10 +28341,10 @@
         <v>Thermowood facade cladding, battens and sunshade profiles with enhanced durability and dimensional stability.</v>
       </c>
       <c r="N527" t="str">
-        <v>(none)</v>
+        <v>/images/products/nordwood/wall-cladding/novawood-wall-cladding-cladding-nova-kd-iroko-cladding.jpg</v>
       </c>
       <c r="O527" t="str">
-        <v/>
+        <v>/images/products/nordwood/wall-cladding/novawood-wall-cladding-cladding-nova-kd-iroko-cladding.jpg</v>
       </c>
       <c r="P527" t="str">
         <v>/products/nordwood/facade?product=facade-facade-cladding-nova-kd-iroko-cladding</v>
@@ -28447,10 +28447,10 @@
         <v>Stair treads and risers in exotic hardwood with brass nosing strips.</v>
       </c>
       <c r="N529" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-01.jpg</v>
       </c>
       <c r="O529" t="str">
-        <v/>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-01.jpg</v>
       </c>
       <c r="P529" t="str">
         <v>/products/heatwood/stairs?product=stairs-aurum-stars-stair-collection-aurum-stars-mo-st-01-mo-st-01</v>
@@ -28500,10 +28500,10 @@
         <v>Stair treads and risers in exotic hardwood with brass nosing strips.</v>
       </c>
       <c r="N530" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-02.jpg</v>
       </c>
       <c r="O530" t="str">
-        <v/>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-02.jpg</v>
       </c>
       <c r="P530" t="str">
         <v>/products/heatwood/stairs?product=stairs-aurum-stars-stair-collection-aurum-stars-mo-st-02-mo-st-02</v>
@@ -28553,10 +28553,10 @@
         <v>Stair treads and risers in exotic hardwood with brass nosing strips.</v>
       </c>
       <c r="N531" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-03.jpg</v>
       </c>
       <c r="O531" t="str">
-        <v/>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-03.jpg</v>
       </c>
       <c r="P531" t="str">
         <v>/products/heatwood/stairs?product=stairs-aurum-stars-stair-collection-aurum-stars-mo-st-03-mo-st-03</v>
@@ -28606,10 +28606,10 @@
         <v>Stair treads and risers in exotic hardwood with brass nosing strips.</v>
       </c>
       <c r="N532" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-04.jpg</v>
       </c>
       <c r="O532" t="str">
-        <v/>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-04.jpg</v>
       </c>
       <c r="P532" t="str">
         <v>/products/heatwood/stairs?product=stairs-aurum-stars-stair-collection-aurum-stars-mo-st-04-mo-st-04</v>
@@ -28659,10 +28659,10 @@
         <v>Stair treads and risers in exotic hardwood with brass nosing strips.</v>
       </c>
       <c r="N533" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-05.jpg</v>
       </c>
       <c r="O533" t="str">
-        <v/>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-05.jpg</v>
       </c>
       <c r="P533" t="str">
         <v>/products/heatwood/stairs?product=stairs-aurum-stars-stair-collection-aurum-stars-mo-st-05-mo-st-05</v>
@@ -28712,10 +28712,10 @@
         <v>Stair treads and risers in exotic hardwood with brass nosing strips.</v>
       </c>
       <c r="N534" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-06.jpg</v>
       </c>
       <c r="O534" t="str">
-        <v/>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-06.jpg</v>
       </c>
       <c r="P534" t="str">
         <v>/products/heatwood/stairs?product=stairs-aurum-stars-stair-collection-aurum-stars-mo-st-06-mo-st-06</v>
@@ -28765,10 +28765,10 @@
         <v>Stair treads and risers in exotic hardwood with brass nosing strips.</v>
       </c>
       <c r="N535" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-07.jpg</v>
       </c>
       <c r="O535" t="str">
-        <v/>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-07.jpg</v>
       </c>
       <c r="P535" t="str">
         <v>/products/heatwood/stairs?product=stairs-aurum-stars-stair-collection-aurum-stars-mo-st-07-mo-st-07</v>
@@ -28818,10 +28818,10 @@
         <v>Stair treads and risers in exotic hardwood with brass nosing strips.</v>
       </c>
       <c r="N536" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-08.jpg</v>
       </c>
       <c r="O536" t="str">
-        <v/>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-08.jpg</v>
       </c>
       <c r="P536" t="str">
         <v>/products/heatwood/stairs?product=stairs-aurum-stars-stair-collection-aurum-stars-mo-st-08-mo-st-08</v>
@@ -28871,10 +28871,10 @@
         <v>Stair treads and risers in exotic hardwood with brass nosing strips.</v>
       </c>
       <c r="N537" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-09.jpg</v>
       </c>
       <c r="O537" t="str">
-        <v/>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-09.jpg</v>
       </c>
       <c r="P537" t="str">
         <v>/products/heatwood/stairs?product=stairs-aurum-stars-stair-collection-aurum-stars-mo-st-09-mo-st-09</v>
@@ -28924,10 +28924,10 @@
         <v>Stair treads and risers in exotic hardwood with brass nosing strips.</v>
       </c>
       <c r="N538" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-10.jpg</v>
       </c>
       <c r="O538" t="str">
-        <v/>
+        <v>/images/products/heatwood/stairs/heatwood-mo-st-10.jpg</v>
       </c>
       <c r="P538" t="str">
         <v>/products/heatwood/stairs?product=stairs-aurum-stars-stair-collection-aurum-stars-mo-st-10-mo-st-10</v>
@@ -28977,10 +28977,10 @@
         <v>Inlay parquet panels with a 3 mm hardwood top layer and natural marble or brass inlays.</v>
       </c>
       <c r="N539" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am106.jpg</v>
       </c>
       <c r="O539" t="str">
-        <v/>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am106.jpg, /images/products/heatwood/aurum-mosaico/heatwood-am106-2.jpg</v>
       </c>
       <c r="P539" t="str">
         <v>/products/heatwood/aurum-mosaico?product=aurum-mosaico-aurum-mosaico-parquet-aurum-mosaico-am106-am106</v>
@@ -29030,10 +29030,10 @@
         <v>Inlay parquet panels with a 3 mm hardwood top layer and natural marble or brass inlays.</v>
       </c>
       <c r="N540" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am102.jpg</v>
       </c>
       <c r="O540" t="str">
-        <v/>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am102.jpg, /images/products/heatwood/aurum-mosaico/heatwood-am102-2.jpg</v>
       </c>
       <c r="P540" t="str">
         <v>/products/heatwood/aurum-mosaico?product=aurum-mosaico-aurum-mosaico-parquet-aurum-mosaico-am102-am102</v>
@@ -29083,10 +29083,10 @@
         <v>Inlay parquet panels with a 3 mm hardwood top layer and natural marble or brass inlays.</v>
       </c>
       <c r="N541" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am108.jpg</v>
       </c>
       <c r="O541" t="str">
-        <v/>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am108.jpg, /images/products/heatwood/aurum-mosaico/heatwood-am108-2.jpg</v>
       </c>
       <c r="P541" t="str">
         <v>/products/heatwood/aurum-mosaico?product=aurum-mosaico-aurum-mosaico-parquet-aurum-mosaico-am108-am108</v>
@@ -29136,10 +29136,10 @@
         <v>Inlay parquet panels with a 3 mm hardwood top layer and natural marble or brass inlays.</v>
       </c>
       <c r="N542" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am104.jpg</v>
       </c>
       <c r="O542" t="str">
-        <v/>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am104.jpg, /images/products/heatwood/aurum-mosaico/heatwood-am104-2.jpg</v>
       </c>
       <c r="P542" t="str">
         <v>/products/heatwood/aurum-mosaico?product=aurum-mosaico-aurum-mosaico-parquet-aurum-mosaico-am104-am104</v>
@@ -29189,10 +29189,10 @@
         <v>Inlay parquet panels with a 3 mm hardwood top layer and natural marble or brass inlays.</v>
       </c>
       <c r="N543" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am501.jpg</v>
       </c>
       <c r="O543" t="str">
-        <v/>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am501.jpg, /images/products/heatwood/aurum-mosaico/heatwood-am501-2.jpg</v>
       </c>
       <c r="P543" t="str">
         <v>/products/heatwood/aurum-mosaico?product=aurum-mosaico-aurum-mosaico-parquet-aurum-mosaico-am501-am501</v>
@@ -29242,10 +29242,10 @@
         <v>Inlay parquet panels with a 3 mm hardwood top layer and natural marble or brass inlays.</v>
       </c>
       <c r="N544" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am502.jpg</v>
       </c>
       <c r="O544" t="str">
-        <v/>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am502.jpg, /images/products/heatwood/aurum-mosaico/heatwood-am502-2.jpg</v>
       </c>
       <c r="P544" t="str">
         <v>/products/heatwood/aurum-mosaico?product=aurum-mosaico-aurum-mosaico-parquet-aurum-mosaico-am502-am502</v>
@@ -29295,10 +29295,10 @@
         <v>Inlay parquet panels with a 3 mm hardwood top layer and natural marble or brass inlays.</v>
       </c>
       <c r="N545" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am201.jpg</v>
       </c>
       <c r="O545" t="str">
-        <v/>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am201.jpg, /images/products/heatwood/aurum-mosaico/heatwood-am201-2.jpg</v>
       </c>
       <c r="P545" t="str">
         <v>/products/heatwood/aurum-mosaico?product=aurum-mosaico-aurum-mosaico-parquet-aurum-mosaico-am201-am201</v>
@@ -29348,10 +29348,10 @@
         <v>Inlay parquet panels with a 3 mm hardwood top layer and natural marble or brass inlays.</v>
       </c>
       <c r="N546" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am401.jpg</v>
       </c>
       <c r="O546" t="str">
-        <v/>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am401.jpg, /images/products/heatwood/aurum-mosaico/heatwood-am401-2.jpg</v>
       </c>
       <c r="P546" t="str">
         <v>/products/heatwood/aurum-mosaico?product=aurum-mosaico-aurum-mosaico-parquet-aurum-mosaico-am401-am401</v>
@@ -29401,10 +29401,10 @@
         <v>Inlay parquet panels with a 3 mm hardwood top layer and natural marble or brass inlays.</v>
       </c>
       <c r="N547" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am109.jpg</v>
       </c>
       <c r="O547" t="str">
-        <v/>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am109.jpg, /images/products/heatwood/aurum-mosaico/heatwood-am109-2.jpg</v>
       </c>
       <c r="P547" t="str">
         <v>/products/heatwood/aurum-mosaico?product=aurum-mosaico-aurum-mosaico-parquet-aurum-mosaico-am109-am109</v>
@@ -29454,10 +29454,10 @@
         <v>Inlay parquet panels with a 3 mm hardwood top layer and natural marble or brass inlays.</v>
       </c>
       <c r="N548" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am602.jpg</v>
       </c>
       <c r="O548" t="str">
-        <v/>
+        <v>/images/products/heatwood/aurum-mosaico/heatwood-am602.jpg, /images/products/heatwood/aurum-mosaico/heatwood-am602-2.jpg</v>
       </c>
       <c r="P548" t="str">
         <v>/products/heatwood/aurum-mosaico?product=aurum-mosaico-aurum-mosaico-parquet-aurum-mosaico-am602-am602</v>
@@ -29507,10 +29507,10 @@
         <v>Border strips with an exotic hardwood frame, natural marble insert and brass strip.</v>
       </c>
       <c r="N549" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/border/heatwood-am746.jpg</v>
       </c>
       <c r="O549" t="str">
-        <v/>
+        <v>/images/products/heatwood/border/heatwood-am746.jpg</v>
       </c>
       <c r="P549" t="str">
         <v>/products/heatwood/border?product=border-aurum-mosaico-border-border-am746-am746</v>
@@ -29560,10 +29560,10 @@
         <v>Border strips with an exotic hardwood frame, natural marble insert and brass strip.</v>
       </c>
       <c r="N550" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/border/heatwood-sm749.jpg</v>
       </c>
       <c r="O550" t="str">
-        <v/>
+        <v>/images/products/heatwood/border/heatwood-sm749.jpg</v>
       </c>
       <c r="P550" t="str">
         <v>/products/heatwood/border?product=border-aurum-mosaico-border-border-sm749-sm749</v>
@@ -29613,10 +29613,10 @@
         <v>Border strips with an exotic hardwood frame, natural marble insert and brass strip.</v>
       </c>
       <c r="N551" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/border/heatwood-am752.jpg</v>
       </c>
       <c r="O551" t="str">
-        <v/>
+        <v>/images/products/heatwood/border/heatwood-am752.jpg</v>
       </c>
       <c r="P551" t="str">
         <v>/products/heatwood/border?product=border-aurum-mosaico-border-border-am752-am752</v>
@@ -29666,10 +29666,10 @@
         <v>Border strips with an exotic hardwood frame, natural marble insert and brass strip.</v>
       </c>
       <c r="N552" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/border/heatwood-am742.jpg</v>
       </c>
       <c r="O552" t="str">
-        <v/>
+        <v>/images/products/heatwood/border/heatwood-am742.jpg</v>
       </c>
       <c r="P552" t="str">
         <v>/products/heatwood/border?product=border-aurum-mosaico-border-border-am742-am742</v>
@@ -29719,10 +29719,10 @@
         <v>Border strips with an exotic hardwood frame, natural marble insert and brass strip.</v>
       </c>
       <c r="N553" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/border/heatwood-sm737.jpg</v>
       </c>
       <c r="O553" t="str">
-        <v/>
+        <v>/images/products/heatwood/border/heatwood-sm737.jpg</v>
       </c>
       <c r="P553" t="str">
         <v>/products/heatwood/border?product=border-aurum-mosaico-border-border-sm737-sm737</v>
@@ -29772,10 +29772,10 @@
         <v>Border strips with an exotic hardwood frame, natural marble insert and brass strip.</v>
       </c>
       <c r="N554" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/border/heatwood-sm596b.jpg</v>
       </c>
       <c r="O554" t="str">
-        <v/>
+        <v>/images/products/heatwood/border/heatwood-sm596b.jpg</v>
       </c>
       <c r="P554" t="str">
         <v>/products/heatwood/border?product=border-aurum-mosaico-border-border-sm596b-sm596b</v>
@@ -29825,10 +29825,10 @@
         <v>Border strips with an exotic hardwood frame, natural marble insert and brass strip.</v>
       </c>
       <c r="N555" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/border/heatwood-am596a.jpg</v>
       </c>
       <c r="O555" t="str">
-        <v/>
+        <v>/images/products/heatwood/border/heatwood-am596a.jpg</v>
       </c>
       <c r="P555" t="str">
         <v>/products/heatwood/border?product=border-aurum-mosaico-border-border-am596a-am596a</v>
@@ -29878,10 +29878,10 @@
         <v>Border strips with an exotic hardwood frame, natural marble insert and brass strip.</v>
       </c>
       <c r="N556" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/border/heatwood-sm753.jpg</v>
       </c>
       <c r="O556" t="str">
-        <v/>
+        <v>/images/products/heatwood/border/heatwood-sm753.jpg</v>
       </c>
       <c r="P556" t="str">
         <v>/products/heatwood/border?product=border-aurum-mosaico-border-border-sm753-sm753</v>
@@ -29931,10 +29931,10 @@
         <v>Border strips with an exotic hardwood frame, natural marble insert and brass strip.</v>
       </c>
       <c r="N557" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/border/heatwood-sm570.jpg</v>
       </c>
       <c r="O557" t="str">
-        <v/>
+        <v>/images/products/heatwood/border/heatwood-sm570.jpg</v>
       </c>
       <c r="P557" t="str">
         <v>/products/heatwood/border?product=border-aurum-mosaico-border-border-sm570-sm570</v>
@@ -29984,10 +29984,10 @@
         <v>Border strips with an exotic hardwood frame, natural marble insert and brass strip.</v>
       </c>
       <c r="N558" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/border/heatwood-sm744.jpg</v>
       </c>
       <c r="O558" t="str">
-        <v/>
+        <v>/images/products/heatwood/border/heatwood-sm744.jpg</v>
       </c>
       <c r="P558" t="str">
         <v>/products/heatwood/border?product=border-aurum-mosaico-border-border-sm744-sm744</v>
@@ -30037,10 +30037,10 @@
         <v>Border strips with an exotic hardwood frame, natural marble insert and brass strip.</v>
       </c>
       <c r="N559" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/border/heatwood-sm583.jpg</v>
       </c>
       <c r="O559" t="str">
-        <v/>
+        <v>/images/products/heatwood/border/heatwood-sm583.jpg</v>
       </c>
       <c r="P559" t="str">
         <v>/products/heatwood/border?product=border-aurum-mosaico-border-border-sm583-sm583</v>
@@ -30090,10 +30090,10 @@
         <v>Border strips with an exotic hardwood frame, natural marble insert and brass strip.</v>
       </c>
       <c r="N560" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/border/heatwood-sm738.jpg</v>
       </c>
       <c r="O560" t="str">
-        <v/>
+        <v>/images/products/heatwood/border/heatwood-sm738.jpg</v>
       </c>
       <c r="P560" t="str">
         <v>/products/heatwood/border?product=border-aurum-mosaico-border-border-sm738-sm738</v>
@@ -30143,10 +30143,10 @@
         <v>Border strips with an exotic hardwood frame, natural marble insert and brass strip.</v>
       </c>
       <c r="N561" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/border/heatwood-sm574.jpg</v>
       </c>
       <c r="O561" t="str">
-        <v/>
+        <v>/images/products/heatwood/border/heatwood-sm574.jpg</v>
       </c>
       <c r="P561" t="str">
         <v>/products/heatwood/border?product=border-aurum-mosaico-border-border-sm574-sm574</v>
@@ -30196,10 +30196,10 @@
         <v>Border strips with an exotic hardwood frame, natural marble insert and brass strip.</v>
       </c>
       <c r="N562" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/border/heatwood-sm578.jpg</v>
       </c>
       <c r="O562" t="str">
-        <v/>
+        <v>/images/products/heatwood/border/heatwood-sm578.jpg</v>
       </c>
       <c r="P562" t="str">
         <v>/products/heatwood/border?product=border-aurum-mosaico-border-border-sm578-sm578</v>
@@ -30249,10 +30249,10 @@
         <v>Border strips with an exotic hardwood frame, natural marble insert and brass strip.</v>
       </c>
       <c r="N563" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/border/heatwood-sm565.jpg</v>
       </c>
       <c r="O563" t="str">
-        <v/>
+        <v>/images/products/heatwood/border/heatwood-sm565.jpg</v>
       </c>
       <c r="P563" t="str">
         <v>/products/heatwood/border?product=border-aurum-mosaico-border-border-sm565-sm565</v>
@@ -30302,10 +30302,10 @@
         <v>Classic and heritage parquet panels with a 3 mm hardwood top layer on waterproof birch plywood.</v>
       </c>
       <c r="N564" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/classic/heatwood-mo-an801.jpg</v>
       </c>
       <c r="O564" t="str">
-        <v/>
+        <v>/images/products/heatwood/classic/heatwood-mo-an801.jpg</v>
       </c>
       <c r="P564" t="str">
         <v>/products/heatwood/classic?product=classic-classic-heritage-parquet-franz-liszt-mo-an801-mo-an801</v>
@@ -30355,10 +30355,10 @@
         <v>Classic and heritage parquet panels with a 3 mm hardwood top layer on waterproof birch plywood.</v>
       </c>
       <c r="N565" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/classic/heatwood-ta-an801.jpg</v>
       </c>
       <c r="O565" t="str">
-        <v/>
+        <v>/images/products/heatwood/classic/heatwood-ta-an801.jpg</v>
       </c>
       <c r="P565" t="str">
         <v>/products/heatwood/classic?product=classic-classic-heritage-parquet-franz-liszt-ta-an801-ta-an801</v>
@@ -30408,10 +30408,10 @@
         <v>Classic and heritage parquet panels with a 3 mm hardwood top layer on waterproof birch plywood.</v>
       </c>
       <c r="N566" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/classic/heatwood-mo-an201-d.jpg</v>
       </c>
       <c r="O566" t="str">
-        <v/>
+        <v>/images/products/heatwood/classic/heatwood-mo-an201-d.jpg</v>
       </c>
       <c r="P566" t="str">
         <v>/products/heatwood/classic?product=classic-classic-heritage-parquet-vienna-star-mo-an201-d-mo-an201-d</v>
@@ -30461,10 +30461,10 @@
         <v>Classic and heritage parquet panels with a 3 mm hardwood top layer on waterproof birch plywood.</v>
       </c>
       <c r="N567" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/classic/heatwood-mo-an201-l.jpg</v>
       </c>
       <c r="O567" t="str">
-        <v/>
+        <v>/images/products/heatwood/classic/heatwood-mo-an201-l.jpg</v>
       </c>
       <c r="P567" t="str">
         <v>/products/heatwood/classic?product=classic-classic-heritage-parquet-vienna-star-mo-an201-l-mo-an201-l</v>
@@ -30514,10 +30514,10 @@
         <v>Classic and heritage parquet panels with a 3 mm hardwood top layer on waterproof birch plywood.</v>
       </c>
       <c r="N568" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/classic/heatwood-ta-an201-l.jpg</v>
       </c>
       <c r="O568" t="str">
-        <v/>
+        <v>/images/products/heatwood/classic/heatwood-ta-an201-l.jpg</v>
       </c>
       <c r="P568" t="str">
         <v>/products/heatwood/classic?product=classic-classic-heritage-parquet-vienna-star-ta-an201-l-ta-an201-l</v>
@@ -30567,10 +30567,10 @@
         <v>Classic and heritage parquet panels with a 3 mm hardwood top layer on waterproof birch plywood.</v>
       </c>
       <c r="N569" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/classic/heatwood-ta-an201-d.jpg</v>
       </c>
       <c r="O569" t="str">
-        <v/>
+        <v>/images/products/heatwood/classic/heatwood-ta-an201-d.jpg</v>
       </c>
       <c r="P569" t="str">
         <v>/products/heatwood/classic?product=classic-classic-heritage-parquet-vienna-star-ta-an201-d-ta-an201-d</v>
@@ -30620,10 +30620,10 @@
         <v>Classic and heritage parquet panels with a 3 mm hardwood top layer on waterproof birch plywood.</v>
       </c>
       <c r="N570" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/classic/heatwood-mo-an301-l.jpg</v>
       </c>
       <c r="O570" t="str">
-        <v/>
+        <v>/images/products/heatwood/classic/heatwood-mo-an301-l.jpg</v>
       </c>
       <c r="P570" t="str">
         <v>/products/heatwood/classic?product=classic-classic-heritage-parquet-clara-schumann-mo-an301-l-mo-an301-l</v>
@@ -30673,10 +30673,10 @@
         <v>Classic and heritage parquet panels with a 3 mm hardwood top layer on waterproof birch plywood.</v>
       </c>
       <c r="N571" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/classic/heatwood-mo-an301-d.jpg</v>
       </c>
       <c r="O571" t="str">
-        <v/>
+        <v>/images/products/heatwood/classic/heatwood-mo-an301-d.jpg</v>
       </c>
       <c r="P571" t="str">
         <v>/products/heatwood/classic?product=classic-classic-heritage-parquet-clara-schumann-mo-an301-d-mo-an301-d</v>
@@ -30726,10 +30726,10 @@
         <v>Classic and heritage parquet panels with a 3 mm hardwood top layer on waterproof birch plywood.</v>
       </c>
       <c r="N572" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/classic/heatwood-mo-f01.jpg</v>
       </c>
       <c r="O572" t="str">
-        <v/>
+        <v>/images/products/heatwood/classic/heatwood-mo-f01.jpg, /images/products/heatwood/classic/heatwood-mo-f01-2.jpg</v>
       </c>
       <c r="P572" t="str">
         <v>/products/heatwood/classic?product=classic-classic-heritage-parquet-santos-rosewood-plank-mo-f01-mo-f01</v>
@@ -30779,10 +30779,10 @@
         <v>Classic and heritage parquet panels with a 3 mm hardwood top layer on waterproof birch plywood.</v>
       </c>
       <c r="N573" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/classic/heatwood-mo-am107-green.jpg</v>
       </c>
       <c r="O573" t="str">
-        <v/>
+        <v>/images/products/heatwood/classic/heatwood-mo-am107-green.jpg</v>
       </c>
       <c r="P573" t="str">
         <v>/products/heatwood/classic?product=classic-classic-heritage-parquet-nicolay-rubinstein-green-marble-mo-am107-mo-am107</v>
@@ -30832,10 +30832,10 @@
         <v>Classic and heritage parquet panels with a 3 mm hardwood top layer on waterproof birch plywood.</v>
       </c>
       <c r="N574" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/classic/heatwood-mo-am107-white.jpg</v>
       </c>
       <c r="O574" t="str">
-        <v/>
+        <v>/images/products/heatwood/classic/heatwood-mo-am107-white.jpg</v>
       </c>
       <c r="P574" t="str">
         <v>/products/heatwood/classic?product=classic-classic-heritage-parquet-nicolay-rubinstein-white-marble-mo-am107-mo-am107</v>
@@ -30885,10 +30885,10 @@
         <v>Classic and heritage parquet panels with a 3 mm hardwood top layer on waterproof birch plywood.</v>
       </c>
       <c r="N575" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/classic/heatwood-mo-am107-burgundy.jpg</v>
       </c>
       <c r="O575" t="str">
-        <v/>
+        <v>/images/products/heatwood/classic/heatwood-mo-am107-burgundy.jpg</v>
       </c>
       <c r="P575" t="str">
         <v>/products/heatwood/classic?product=classic-classic-heritage-parquet-nicolay-rubinstein-burgundy-black-marble-mo-am107-mo-am107</v>
@@ -30938,10 +30938,10 @@
         <v>Classic and heritage parquet panels with a 3 mm hardwood top layer on waterproof birch plywood.</v>
       </c>
       <c r="N576" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/classic/heatwood-ta-am107.jpg</v>
       </c>
       <c r="O576" t="str">
-        <v/>
+        <v>/images/products/heatwood/classic/heatwood-ta-am107.jpg</v>
       </c>
       <c r="P576" t="str">
         <v>/products/heatwood/classic?product=classic-classic-heritage-parquet-nicolay-rubinstein-simple-elegant-luxury-ta-am107-ta-am107</v>
@@ -30991,10 +30991,10 @@
         <v>Classic and heritage parquet panels with a 3 mm hardwood top layer on waterproof birch plywood.</v>
       </c>
       <c r="N577" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/classic/heatwood-mo-co1.jpg</v>
       </c>
       <c r="O577" t="str">
-        <v/>
+        <v>/images/products/heatwood/classic/heatwood-mo-co1.jpg, /images/products/heatwood/classic/heatwood-mo-co1-2.jpg</v>
       </c>
       <c r="P577" t="str">
         <v>/products/heatwood/classic?product=classic-classic-heritage-parquet-chevron-mo-co1-mo-co1</v>
@@ -31044,10 +31044,10 @@
         <v>Classic and heritage parquet panels with a 3 mm hardwood top layer on waterproof birch plywood.</v>
       </c>
       <c r="N578" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/classic/heatwood-mo-h01.jpg</v>
       </c>
       <c r="O578" t="str">
-        <v/>
+        <v>/images/products/heatwood/classic/heatwood-mo-h01.jpg</v>
       </c>
       <c r="P578" t="str">
         <v>/products/heatwood/classic?product=classic-classic-heritage-parquet-herringbone-mo-h01-mo-h01</v>
@@ -31097,10 +31097,10 @@
         <v>Classic and heritage parquet panels with a 3 mm hardwood top layer on waterproof birch plywood.</v>
       </c>
       <c r="N579" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/classic/heatwood-sm-60.jpg</v>
       </c>
       <c r="O579" t="str">
-        <v/>
+        <v>/images/products/heatwood/classic/heatwood-sm-60.jpg</v>
       </c>
       <c r="P579" t="str">
         <v>/products/heatwood/classic?product=classic-classic-heritage-parquet-heritage-panel-sm-60-sm-60</v>
@@ -31203,10 +31203,10 @@
         <v>Classic and heritage parquet panels with a 3 mm hardwood top layer on waterproof birch plywood.</v>
       </c>
       <c r="N581" t="str">
-        <v>(none)</v>
+        <v>/images/products/heatwood/classic/heatwood-sm-518.jpg</v>
       </c>
       <c r="O581" t="str">
-        <v/>
+        <v>/images/products/heatwood/classic/heatwood-sm-518.jpg</v>
       </c>
       <c r="P581" t="str">
         <v>/products/heatwood/classic?product=classic-classic-heritage-parquet-imperium-carved-panel-sm-518-sm-518</v>
@@ -31265,7 +31265,7 @@
         <v>149</v>
       </c>
       <c r="E2">
-        <v>45</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3">
@@ -31299,7 +31299,7 @@
         <v>18</v>
       </c>
       <c r="E4">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -31316,7 +31316,7 @@
         <v>105</v>
       </c>
       <c r="E5">
-        <v>13</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6">
@@ -31367,7 +31367,7 @@
         <v>17</v>
       </c>
       <c r="E8">
-        <v>5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
@@ -31384,7 +31384,7 @@
         <v>30</v>
       </c>
       <c r="E9">
-        <v>14</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10">
@@ -31401,7 +31401,7 @@
         <v>45</v>
       </c>
       <c r="E10">
-        <v>7</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11">
@@ -31418,7 +31418,7 @@
         <v>21</v>
       </c>
       <c r="E11">
-        <v>9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12">
@@ -31452,7 +31452,7 @@
         <v>10</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -31469,7 +31469,7 @@
         <v>10</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
@@ -31486,7 +31486,7 @@
         <v>15</v>
       </c>
       <c r="E15">
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16">
@@ -31503,7 +31503,7 @@
         <v>18</v>
       </c>
       <c r="E16">
-        <v>0</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17">
@@ -31520,7 +31520,7 @@
         <v>580</v>
       </c>
       <c r="E17">
-        <v>249</v>
+        <v>572</v>
       </c>
     </row>
   </sheetData>

</xml_diff>